<commit_message>
chore: sync all workspace files
Task-ID: workspace-sync-20260822
</commit_message>
<xml_diff>
--- a/data_assets/mapping/dwd_to_dws/DWS汇总层数据模型_CRM_ V1.0.xlsx
+++ b/data_assets/mapping/dwd_to_dws/DWS汇总层数据模型_CRM_ V1.0.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr codeName="ThisWorkbook"/>
   <bookViews>
-    <workbookView windowWidth="22188" windowHeight="9060" tabRatio="753" firstSheet="5" activeTab="9"/>
+    <workbookView windowWidth="22188" windowHeight="9060" tabRatio="753" firstSheet="5" activeTab="10"/>
   </bookViews>
   <sheets>
     <sheet name="修订记录" sheetId="1" r:id="rId1"/>
@@ -17,17 +17,18 @@
     <sheet name="客户转介绍" sheetId="8" r:id="rId8"/>
     <sheet name="转介绍提醒表" sheetId="9" r:id="rId9"/>
     <sheet name="客户资产负债基数表" sheetId="10" r:id="rId10"/>
-    <sheet name="客户资产负债表" sheetId="11" r:id="rId11"/>
-    <sheet name="客户等级信息表" sheetId="12" r:id="rId12"/>
-    <sheet name="零售潜在客户信息表" sheetId="13" r:id="rId13"/>
-    <sheet name="逻辑模型维度描述" sheetId="14" state="hidden" r:id="rId14"/>
+    <sheet name="客户资产负债表历史表" sheetId="15" r:id="rId11"/>
+    <sheet name="客户资产负债表" sheetId="11" r:id="rId12"/>
+    <sheet name="客户等级信息表" sheetId="12" r:id="rId13"/>
+    <sheet name="零售潜在客户信息表" sheetId="13" r:id="rId14"/>
+    <sheet name="逻辑模型维度描述" sheetId="14" state="hidden" r:id="rId15"/>
   </sheets>
   <externalReferences>
-    <externalReference r:id="rId15"/>
     <externalReference r:id="rId16"/>
     <externalReference r:id="rId17"/>
     <externalReference r:id="rId18"/>
     <externalReference r:id="rId19"/>
+    <externalReference r:id="rId20"/>
   </externalReferences>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">实体清单!$B$1:$G$8</definedName>
@@ -53,17 +54,6 @@
     <definedName name="_Toc205004289" localSheetId="9">#REF!</definedName>
     <definedName name="_Toc275247984" localSheetId="9">#REF!</definedName>
     <definedName name="Basel" localSheetId="9">[2]Parameters!$C$32:$C$33</definedName>
-    <definedName name="Database" localSheetId="10" hidden="1">#REF!</definedName>
-    <definedName name="_Toc205004290" localSheetId="10">#REF!</definedName>
-    <definedName name="常用数据标准" localSheetId="10">#REF!</definedName>
-    <definedName name="_Toc205004288" localSheetId="10">#REF!</definedName>
-    <definedName name="_Toc256075879" localSheetId="10">#REF!</definedName>
-    <definedName name="YesNoBasel2" localSheetId="10">[3]Parameters!#REF!</definedName>
-    <definedName name="area" localSheetId="10">[1]建议意见清单!$A$1:$F$21</definedName>
-    <definedName name="_Toc205004291" localSheetId="10">#REF!</definedName>
-    <definedName name="_Toc205004289" localSheetId="10">#REF!</definedName>
-    <definedName name="_Toc275247984" localSheetId="10">#REF!</definedName>
-    <definedName name="Basel" localSheetId="10">[2]Parameters!$C$32:$C$33</definedName>
     <definedName name="Database" localSheetId="11" hidden="1">#REF!</definedName>
     <definedName name="_Toc205004290" localSheetId="11">#REF!</definedName>
     <definedName name="常用数据标准" localSheetId="11">#REF!</definedName>
@@ -80,12 +70,34 @@
     <definedName name="常用数据标准" localSheetId="12">#REF!</definedName>
     <definedName name="_Toc205004288" localSheetId="12">#REF!</definedName>
     <definedName name="_Toc256075879" localSheetId="12">#REF!</definedName>
-    <definedName name="YesNoBasel2" localSheetId="12">[5]Parameters!#REF!</definedName>
+    <definedName name="YesNoBasel2" localSheetId="12">[3]Parameters!#REF!</definedName>
     <definedName name="area" localSheetId="12">[1]建议意见清单!$A$1:$F$21</definedName>
     <definedName name="_Toc205004291" localSheetId="12">#REF!</definedName>
     <definedName name="_Toc205004289" localSheetId="12">#REF!</definedName>
     <definedName name="_Toc275247984" localSheetId="12">#REF!</definedName>
-    <definedName name="Basel" localSheetId="12">[4]Parameters!$C$32:$C$33</definedName>
+    <definedName name="Basel" localSheetId="12">[2]Parameters!$C$32:$C$33</definedName>
+    <definedName name="Database" localSheetId="13" hidden="1">#REF!</definedName>
+    <definedName name="_Toc205004290" localSheetId="13">#REF!</definedName>
+    <definedName name="常用数据标准" localSheetId="13">#REF!</definedName>
+    <definedName name="_Toc205004288" localSheetId="13">#REF!</definedName>
+    <definedName name="_Toc256075879" localSheetId="13">#REF!</definedName>
+    <definedName name="YesNoBasel2" localSheetId="13">[5]Parameters!#REF!</definedName>
+    <definedName name="area" localSheetId="13">[1]建议意见清单!$A$1:$F$21</definedName>
+    <definedName name="_Toc205004291" localSheetId="13">#REF!</definedName>
+    <definedName name="_Toc205004289" localSheetId="13">#REF!</definedName>
+    <definedName name="_Toc275247984" localSheetId="13">#REF!</definedName>
+    <definedName name="Basel" localSheetId="13">[4]Parameters!$C$32:$C$33</definedName>
+    <definedName name="Database" localSheetId="10" hidden="1">#REF!</definedName>
+    <definedName name="_Toc205004290" localSheetId="10">#REF!</definedName>
+    <definedName name="常用数据标准" localSheetId="10">#REF!</definedName>
+    <definedName name="_Toc205004288" localSheetId="10">#REF!</definedName>
+    <definedName name="_Toc256075879" localSheetId="10">#REF!</definedName>
+    <definedName name="YesNoBasel2" localSheetId="10">[3]Parameters!#REF!</definedName>
+    <definedName name="area" localSheetId="10">[1]建议意见清单!$A$1:$F$21</definedName>
+    <definedName name="_Toc205004291" localSheetId="10">#REF!</definedName>
+    <definedName name="_Toc205004289" localSheetId="10">#REF!</definedName>
+    <definedName name="_Toc275247984" localSheetId="10">#REF!</definedName>
+    <definedName name="Basel" localSheetId="10">[2]Parameters!$C$32:$C$33</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -105,7 +117,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1479" uniqueCount="442">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1567" uniqueCount="444">
   <si>
     <t>文档修订记录</t>
   </si>
@@ -840,100 +852,106 @@
     <t>投保单号或者借据号</t>
   </si>
   <si>
+    <t>客户资产负债表历史表</t>
+  </si>
+  <si>
+    <t>DWS_CUST_ASSE_LIAB_HIS</t>
+  </si>
+  <si>
+    <t>ORG_ID_LOAN</t>
+  </si>
+  <si>
+    <t>信贷归属机构</t>
+  </si>
+  <si>
+    <t>BAL_TYPE</t>
+  </si>
+  <si>
+    <t>类型1-余额2-月日均3-季日均4-年日均</t>
+  </si>
+  <si>
+    <t>AUM_BAL</t>
+  </si>
+  <si>
+    <t>AUM余额</t>
+  </si>
+  <si>
+    <t>DEPO_BAL</t>
+  </si>
+  <si>
+    <t>存款余额</t>
+  </si>
+  <si>
+    <t>DEPO_CURNT_DEPO_BAL</t>
+  </si>
+  <si>
+    <t>活期余额</t>
+  </si>
+  <si>
+    <t>FIXD_DEPO_BAL</t>
+  </si>
+  <si>
+    <t>普通定期余额</t>
+  </si>
+  <si>
+    <t>LEHUI_BAL</t>
+  </si>
+  <si>
+    <t>乐惠存产品余额</t>
+  </si>
+  <si>
+    <t>LARGEDP_BAL</t>
+  </si>
+  <si>
+    <t>大额存单余额</t>
+  </si>
+  <si>
+    <t>FIN_BAL</t>
+  </si>
+  <si>
+    <t>理财余额</t>
+  </si>
+  <si>
+    <t>CLOSE_AGEN_FIN_BAL</t>
+  </si>
+  <si>
+    <t>代销封闭式理财余额</t>
+  </si>
+  <si>
+    <t>OPEN_AGEN_FIN_BAL</t>
+  </si>
+  <si>
+    <t>代销开放式理财余额</t>
+  </si>
+  <si>
+    <t>CLOSE_SELF_FIN_BAL</t>
+  </si>
+  <si>
+    <t>自营封闭式理财余额</t>
+  </si>
+  <si>
+    <t>OPEN_SELF_FIN_BAL</t>
+  </si>
+  <si>
+    <t>自营开放式理财余额</t>
+  </si>
+  <si>
+    <t>INSUR_BAL</t>
+  </si>
+  <si>
+    <t>保险余额</t>
+  </si>
+  <si>
+    <t>LOAN_BAL</t>
+  </si>
+  <si>
+    <t>贷款余额</t>
+  </si>
+  <si>
     <t>客户资产负债表</t>
   </si>
   <si>
     <t>DWS_CUST_ASSE_LIAB</t>
-  </si>
-  <si>
-    <t>ORG_ID_LOAN</t>
-  </si>
-  <si>
-    <t>信贷归属机构</t>
-  </si>
-  <si>
-    <t>BAL_TYPE</t>
-  </si>
-  <si>
-    <t>类型1-余额2-月日均3-季日均4-年日均</t>
-  </si>
-  <si>
-    <t>AUM_BAL</t>
-  </si>
-  <si>
-    <t>AUM余额</t>
-  </si>
-  <si>
-    <t>DEPO_BAL</t>
-  </si>
-  <si>
-    <t>定期余额</t>
-  </si>
-  <si>
-    <t>DEPO_CURNT_DEPO_BAL</t>
-  </si>
-  <si>
-    <t>活期余额</t>
-  </si>
-  <si>
-    <t>FIXD_DEPO_BAL</t>
-  </si>
-  <si>
-    <t>普通定期余额</t>
-  </si>
-  <si>
-    <t>LEHUI_BAL</t>
-  </si>
-  <si>
-    <t>乐惠存产品余额</t>
-  </si>
-  <si>
-    <t>LARGEDP_BAL</t>
-  </si>
-  <si>
-    <t>大额存单余额</t>
-  </si>
-  <si>
-    <t>FIN_BAL</t>
-  </si>
-  <si>
-    <t>理财余额</t>
-  </si>
-  <si>
-    <t>CLOSE_AGEN_FIN_BAL</t>
-  </si>
-  <si>
-    <t>代销封闭式理财余额</t>
-  </si>
-  <si>
-    <t>OPEN_AGEN_FIN_BAL</t>
-  </si>
-  <si>
-    <t>代销开放式理财余额</t>
-  </si>
-  <si>
-    <t>CLOSE_SELF_FIN_BAL</t>
-  </si>
-  <si>
-    <t>自营封闭式理财余额</t>
-  </si>
-  <si>
-    <t>OPEN_SELF_FIN_BAL</t>
-  </si>
-  <si>
-    <t>自营开放式理财余额</t>
-  </si>
-  <si>
-    <t>INSUR_BAL</t>
-  </si>
-  <si>
-    <t>保险余额</t>
-  </si>
-  <si>
-    <t>LOAN_BAL</t>
-  </si>
-  <si>
-    <t>贷款余额</t>
   </si>
   <si>
     <t>客户等级信息表</t>
@@ -6102,7 +6120,7 @@
     <mergeCell ref="L40:Q40"/>
   </mergeCells>
   <dataValidations count="1">
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="C21 C22 C23 C7:C8">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="C7:C8 C21:C23">
       <formula1>#REF!</formula1>
     </dataValidation>
   </dataValidations>
@@ -6918,6 +6936,810 @@
 <file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
+  <dimension ref="A1:Q83"/>
+  <sheetFormatPr defaultColWidth="8.23148148148148" defaultRowHeight="14.4"/>
+  <cols>
+    <col min="1" max="1" width="9.66666666666667" style="70" customWidth="1"/>
+    <col min="2" max="2" width="27.5462962962963" style="70" customWidth="1"/>
+    <col min="3" max="3" width="8.88888888888889" style="70" customWidth="1"/>
+    <col min="4" max="4" width="15.1851851851852" style="70" customWidth="1"/>
+    <col min="5" max="5" width="38.8888888888889" style="70" customWidth="1"/>
+    <col min="6" max="6" width="10.7685185185185" style="70" customWidth="1"/>
+    <col min="7" max="7" width="12.1018518518519" style="70" customWidth="1"/>
+    <col min="8" max="8" width="8.76851851851852" style="70" customWidth="1"/>
+    <col min="9" max="9" width="8.23148148148148" style="70" customWidth="1"/>
+    <col min="10" max="10" width="8.76851851851852" style="70" customWidth="1"/>
+    <col min="11" max="11" width="8.23148148148148" style="70" customWidth="1"/>
+    <col min="12" max="12" width="24.1851851851852" style="70" customWidth="1"/>
+    <col min="13" max="13" width="23" style="70" customWidth="1"/>
+    <col min="14" max="14" width="17.3611111111111" style="70" customWidth="1"/>
+    <col min="15" max="15" width="16.8796296296296" style="70" customWidth="1"/>
+    <col min="16" max="16" width="10.2685185185185" style="70" customWidth="1"/>
+    <col min="17" max="17" width="16.8148148148148" style="70" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" s="3" customFormat="1" ht="17.4" customHeight="1" spans="1:17">
+      <c r="B1" s="71" t="s">
+        <v>27</v>
+      </c>
+      <c r="C1" s="72"/>
+      <c r="D1" s="72"/>
+      <c r="E1" s="72"/>
+      <c r="F1" s="72"/>
+      <c r="G1" s="72"/>
+      <c r="H1" s="72"/>
+      <c r="I1" s="72"/>
+      <c r="J1" s="72"/>
+    </row>
+    <row r="2" s="3" customFormat="1" ht="21" customHeight="1" spans="1:17">
+      <c r="B2" s="73" t="s">
+        <v>16</v>
+      </c>
+      <c r="C2" s="74" t="s">
+        <v>274</v>
+      </c>
+      <c r="D2" s="12"/>
+      <c r="E2" s="12"/>
+      <c r="F2" s="75" t="s">
+        <v>275</v>
+      </c>
+      <c r="G2" s="12"/>
+      <c r="H2" s="12"/>
+      <c r="I2" s="12"/>
+      <c r="J2" s="13"/>
+    </row>
+    <row r="3" s="3" customFormat="1" ht="30.6" customHeight="1" spans="1:17">
+      <c r="B3" s="11"/>
+      <c r="C3" s="12"/>
+      <c r="D3" s="12"/>
+      <c r="E3" s="12"/>
+      <c r="F3" s="12"/>
+      <c r="G3" s="12"/>
+      <c r="H3" s="12"/>
+      <c r="I3" s="12"/>
+      <c r="J3" s="13"/>
+    </row>
+    <row r="4" s="3" customFormat="1" ht="17.55" customHeight="1" spans="1:17">
+      <c r="B4" s="76" t="s">
+        <v>30</v>
+      </c>
+      <c r="C4" s="12"/>
+      <c r="D4" s="12"/>
+      <c r="E4" s="12"/>
+      <c r="F4" s="12"/>
+      <c r="G4" s="12"/>
+      <c r="H4" s="12"/>
+      <c r="I4" s="12"/>
+      <c r="J4" s="13"/>
+      <c r="L4" s="77" t="s">
+        <v>31</v>
+      </c>
+      <c r="M4" s="39"/>
+      <c r="N4" s="39"/>
+      <c r="O4" s="39"/>
+      <c r="P4" s="39"/>
+      <c r="Q4" s="40"/>
+    </row>
+    <row r="5" s="4" customFormat="1" ht="16.95" customHeight="1" spans="1:17">
+      <c r="B5" s="78" t="s">
+        <v>32</v>
+      </c>
+      <c r="C5" s="78" t="s">
+        <v>33</v>
+      </c>
+      <c r="D5" s="78" t="s">
+        <v>34</v>
+      </c>
+      <c r="E5" s="78" t="s">
+        <v>35</v>
+      </c>
+      <c r="F5" s="78" t="s">
+        <v>36</v>
+      </c>
+      <c r="G5" s="13"/>
+      <c r="H5" s="78" t="s">
+        <v>37</v>
+      </c>
+      <c r="I5" s="79" t="s">
+        <v>38</v>
+      </c>
+      <c r="J5" s="79" t="s">
+        <v>39</v>
+      </c>
+      <c r="L5" s="22" t="s">
+        <v>40</v>
+      </c>
+      <c r="M5" s="23" t="s">
+        <v>41</v>
+      </c>
+      <c r="N5" s="23" t="s">
+        <v>42</v>
+      </c>
+      <c r="O5" s="23" t="s">
+        <v>43</v>
+      </c>
+      <c r="P5" s="23" t="s">
+        <v>44</v>
+      </c>
+      <c r="Q5" s="24" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="6" s="6" customFormat="1" ht="13.95" customHeight="1" spans="1:17">
+      <c r="A6" s="80"/>
+      <c r="B6" s="81" t="s">
+        <v>137</v>
+      </c>
+      <c r="C6" s="82"/>
+      <c r="D6" s="81" t="s">
+        <v>138</v>
+      </c>
+      <c r="E6" s="81" t="s">
+        <v>139</v>
+      </c>
+      <c r="F6" s="83"/>
+      <c r="G6" s="83"/>
+      <c r="H6" s="84"/>
+      <c r="I6" s="85"/>
+      <c r="J6" s="86"/>
+      <c r="L6" s="87"/>
+      <c r="M6" s="81"/>
+      <c r="N6" s="87"/>
+      <c r="O6" s="87"/>
+      <c r="P6" s="88"/>
+      <c r="Q6" s="88"/>
+    </row>
+    <row r="7" s="6" customFormat="1" ht="13.95" customHeight="1" spans="1:17">
+      <c r="A7" s="80"/>
+      <c r="B7" s="81" t="s">
+        <v>61</v>
+      </c>
+      <c r="C7" s="82"/>
+      <c r="D7" s="81" t="s">
+        <v>56</v>
+      </c>
+      <c r="E7" s="81" t="s">
+        <v>213</v>
+      </c>
+      <c r="F7" s="83"/>
+      <c r="G7" s="83"/>
+      <c r="H7" s="84"/>
+      <c r="I7" s="85"/>
+      <c r="J7" s="86"/>
+      <c r="L7" s="87"/>
+      <c r="M7" s="81"/>
+      <c r="N7" s="87"/>
+      <c r="O7" s="87"/>
+      <c r="P7" s="88"/>
+      <c r="Q7" s="88"/>
+    </row>
+    <row r="8" s="6" customFormat="1" ht="13.95" customHeight="1" spans="1:17">
+      <c r="A8" s="80"/>
+      <c r="B8" s="81" t="s">
+        <v>76</v>
+      </c>
+      <c r="C8" s="82"/>
+      <c r="D8" s="81" t="s">
+        <v>77</v>
+      </c>
+      <c r="E8" s="81" t="s">
+        <v>212</v>
+      </c>
+      <c r="F8" s="83"/>
+      <c r="G8" s="83"/>
+      <c r="H8" s="84"/>
+      <c r="I8" s="85"/>
+      <c r="J8" s="86"/>
+      <c r="L8" s="87"/>
+      <c r="M8" s="81"/>
+      <c r="N8" s="87"/>
+      <c r="O8" s="90"/>
+      <c r="P8" s="88"/>
+      <c r="Q8" s="88"/>
+    </row>
+    <row r="9" s="6" customFormat="1" ht="13.95" customHeight="1" spans="1:17">
+      <c r="A9" s="80"/>
+      <c r="B9" s="81" t="s">
+        <v>244</v>
+      </c>
+      <c r="C9" s="82"/>
+      <c r="D9" s="81" t="s">
+        <v>50</v>
+      </c>
+      <c r="E9" s="81" t="s">
+        <v>245</v>
+      </c>
+      <c r="F9" s="83"/>
+      <c r="G9" s="83"/>
+      <c r="H9" s="84"/>
+      <c r="I9" s="85"/>
+      <c r="J9" s="86"/>
+      <c r="L9" s="87"/>
+      <c r="M9" s="81"/>
+      <c r="N9" s="87"/>
+      <c r="O9" s="87"/>
+      <c r="P9" s="88"/>
+      <c r="Q9" s="88"/>
+    </row>
+    <row r="10" s="6" customFormat="1" ht="13.95" customHeight="1" spans="1:17">
+      <c r="A10" s="80"/>
+      <c r="B10" s="81" t="s">
+        <v>246</v>
+      </c>
+      <c r="C10" s="82"/>
+      <c r="D10" s="81" t="s">
+        <v>90</v>
+      </c>
+      <c r="E10" s="81" t="s">
+        <v>247</v>
+      </c>
+      <c r="F10" s="83"/>
+      <c r="G10" s="83"/>
+      <c r="H10" s="84"/>
+      <c r="I10" s="85"/>
+      <c r="J10" s="86"/>
+      <c r="L10" s="87"/>
+      <c r="M10" s="81"/>
+      <c r="N10" s="87"/>
+      <c r="O10" s="87"/>
+      <c r="P10" s="88"/>
+      <c r="Q10" s="88"/>
+    </row>
+    <row r="11" s="6" customFormat="1" ht="13.95" customHeight="1" spans="1:17">
+      <c r="A11" s="80"/>
+      <c r="B11" s="81" t="s">
+        <v>248</v>
+      </c>
+      <c r="C11" s="82"/>
+      <c r="D11" s="81" t="s">
+        <v>70</v>
+      </c>
+      <c r="E11" s="81" t="s">
+        <v>249</v>
+      </c>
+      <c r="F11" s="83"/>
+      <c r="G11" s="83"/>
+      <c r="H11" s="84"/>
+      <c r="I11" s="85"/>
+      <c r="J11" s="86"/>
+      <c r="L11" s="87"/>
+      <c r="M11" s="81"/>
+      <c r="N11" s="87"/>
+      <c r="O11" s="87"/>
+      <c r="P11" s="88"/>
+      <c r="Q11" s="88"/>
+    </row>
+    <row r="12" s="6" customFormat="1" ht="13.95" customHeight="1" spans="1:17">
+      <c r="A12" s="80"/>
+      <c r="B12" s="81" t="s">
+        <v>250</v>
+      </c>
+      <c r="C12" s="82"/>
+      <c r="D12" s="81" t="s">
+        <v>70</v>
+      </c>
+      <c r="E12" s="81" t="s">
+        <v>251</v>
+      </c>
+      <c r="F12" s="83"/>
+      <c r="G12" s="83"/>
+      <c r="H12" s="84"/>
+      <c r="I12" s="85"/>
+      <c r="J12" s="86"/>
+      <c r="L12" s="87"/>
+      <c r="M12" s="81"/>
+      <c r="N12" s="87"/>
+      <c r="O12" s="90"/>
+      <c r="P12" s="88"/>
+      <c r="Q12" s="88"/>
+    </row>
+    <row r="13" s="6" customFormat="1" ht="13.95" customHeight="1" spans="1:17">
+      <c r="A13" s="80"/>
+      <c r="B13" s="81" t="s">
+        <v>252</v>
+      </c>
+      <c r="C13" s="82"/>
+      <c r="D13" s="81" t="s">
+        <v>70</v>
+      </c>
+      <c r="E13" s="81" t="s">
+        <v>253</v>
+      </c>
+      <c r="F13" s="83"/>
+      <c r="G13" s="83"/>
+      <c r="H13" s="84"/>
+      <c r="I13" s="85"/>
+      <c r="J13" s="86"/>
+      <c r="L13" s="87"/>
+      <c r="M13" s="81"/>
+      <c r="N13" s="87"/>
+      <c r="O13" s="90"/>
+      <c r="P13" s="88"/>
+      <c r="Q13" s="88"/>
+    </row>
+    <row r="14" s="6" customFormat="1" ht="13.95" customHeight="1" spans="1:17">
+      <c r="A14" s="80"/>
+      <c r="B14" s="81" t="s">
+        <v>254</v>
+      </c>
+      <c r="C14" s="82"/>
+      <c r="D14" s="81" t="s">
+        <v>70</v>
+      </c>
+      <c r="E14" s="81" t="s">
+        <v>255</v>
+      </c>
+      <c r="F14" s="83"/>
+      <c r="G14" s="83"/>
+      <c r="H14" s="84"/>
+      <c r="I14" s="85"/>
+      <c r="J14" s="86"/>
+      <c r="L14" s="87"/>
+      <c r="M14" s="81"/>
+      <c r="N14" s="87"/>
+      <c r="O14" s="90"/>
+      <c r="P14" s="88"/>
+      <c r="Q14" s="88"/>
+    </row>
+    <row r="15" s="6" customFormat="1" ht="13.95" customHeight="1" spans="1:17">
+      <c r="A15" s="80"/>
+      <c r="B15" s="81" t="s">
+        <v>256</v>
+      </c>
+      <c r="C15" s="82"/>
+      <c r="D15" s="81" t="s">
+        <v>70</v>
+      </c>
+      <c r="E15" s="81" t="s">
+        <v>257</v>
+      </c>
+      <c r="F15" s="83"/>
+      <c r="G15" s="83"/>
+      <c r="H15" s="84"/>
+      <c r="I15" s="85"/>
+      <c r="J15" s="86"/>
+      <c r="L15" s="87"/>
+      <c r="M15" s="81"/>
+      <c r="N15" s="87"/>
+      <c r="O15" s="87"/>
+      <c r="P15" s="88"/>
+      <c r="Q15" s="88"/>
+    </row>
+    <row r="16" s="6" customFormat="1" ht="13.95" customHeight="1" spans="1:17">
+      <c r="A16" s="80"/>
+      <c r="B16" s="81" t="s">
+        <v>258</v>
+      </c>
+      <c r="C16" s="82"/>
+      <c r="D16" s="81" t="s">
+        <v>70</v>
+      </c>
+      <c r="E16" s="81" t="s">
+        <v>259</v>
+      </c>
+      <c r="F16" s="83"/>
+      <c r="G16" s="83"/>
+      <c r="H16" s="84"/>
+      <c r="I16" s="85"/>
+      <c r="J16" s="86"/>
+      <c r="L16" s="87"/>
+      <c r="M16" s="81"/>
+      <c r="N16" s="87"/>
+      <c r="O16" s="90"/>
+      <c r="P16" s="88"/>
+      <c r="Q16" s="88"/>
+    </row>
+    <row r="17" s="6" customFormat="1" ht="13.95" customHeight="1" spans="1:17">
+      <c r="A17" s="80"/>
+      <c r="B17" s="81" t="s">
+        <v>260</v>
+      </c>
+      <c r="C17" s="82"/>
+      <c r="D17" s="81" t="s">
+        <v>70</v>
+      </c>
+      <c r="E17" s="81" t="s">
+        <v>261</v>
+      </c>
+      <c r="F17" s="83"/>
+      <c r="G17" s="83"/>
+      <c r="H17" s="84"/>
+      <c r="I17" s="85"/>
+      <c r="J17" s="86"/>
+      <c r="L17" s="87"/>
+      <c r="M17" s="81"/>
+      <c r="N17" s="87"/>
+      <c r="O17" s="87"/>
+      <c r="P17" s="88"/>
+      <c r="Q17" s="88"/>
+    </row>
+    <row r="18" s="6" customFormat="1" ht="13.95" customHeight="1" spans="1:17">
+      <c r="A18" s="80"/>
+      <c r="B18" s="91" t="s">
+        <v>262</v>
+      </c>
+      <c r="C18" s="82"/>
+      <c r="D18" s="81" t="s">
+        <v>70</v>
+      </c>
+      <c r="E18" s="81" t="s">
+        <v>263</v>
+      </c>
+      <c r="F18" s="83"/>
+      <c r="G18" s="83"/>
+      <c r="H18" s="84"/>
+      <c r="I18" s="85"/>
+      <c r="J18" s="86"/>
+    </row>
+    <row r="19" s="6" customFormat="1" ht="13.95" customHeight="1" spans="1:17">
+      <c r="A19" s="80"/>
+      <c r="B19" s="91" t="s">
+        <v>264</v>
+      </c>
+      <c r="C19" s="82"/>
+      <c r="D19" s="81" t="s">
+        <v>70</v>
+      </c>
+      <c r="E19" s="81" t="s">
+        <v>265</v>
+      </c>
+      <c r="F19" s="83"/>
+      <c r="G19" s="83"/>
+      <c r="H19" s="84"/>
+      <c r="I19" s="85"/>
+      <c r="J19" s="86"/>
+    </row>
+    <row r="20" s="6" customFormat="1" ht="13.95" customHeight="1" spans="1:17">
+      <c r="A20" s="80"/>
+      <c r="B20" s="91" t="s">
+        <v>266</v>
+      </c>
+      <c r="C20" s="82"/>
+      <c r="D20" s="81" t="s">
+        <v>70</v>
+      </c>
+      <c r="E20" s="81" t="s">
+        <v>267</v>
+      </c>
+      <c r="F20" s="83"/>
+      <c r="G20" s="83"/>
+      <c r="H20" s="84"/>
+      <c r="I20" s="85"/>
+      <c r="J20" s="86"/>
+    </row>
+    <row r="21" s="3" customFormat="1" ht="17.4" customHeight="1" spans="1:17">
+      <c r="A21" s="80"/>
+      <c r="B21" s="91" t="s">
+        <v>268</v>
+      </c>
+      <c r="C21" s="82"/>
+      <c r="D21" s="81" t="s">
+        <v>70</v>
+      </c>
+      <c r="E21" s="81" t="s">
+        <v>269</v>
+      </c>
+      <c r="F21" s="85"/>
+      <c r="G21" s="85"/>
+      <c r="H21" s="85"/>
+      <c r="I21" s="85"/>
+      <c r="J21" s="85"/>
+    </row>
+    <row r="22" s="3" customFormat="1" ht="17.4" customHeight="1" spans="1:17">
+      <c r="A22" s="80"/>
+      <c r="B22" s="91" t="s">
+        <v>270</v>
+      </c>
+      <c r="C22" s="82"/>
+      <c r="D22" s="81" t="s">
+        <v>70</v>
+      </c>
+      <c r="E22" s="81" t="s">
+        <v>271</v>
+      </c>
+      <c r="F22" s="85"/>
+      <c r="G22" s="85"/>
+      <c r="H22" s="85"/>
+      <c r="I22" s="85"/>
+      <c r="J22" s="85"/>
+      <c r="L22" s="87"/>
+      <c r="M22" s="81"/>
+      <c r="N22" s="87"/>
+      <c r="O22" s="90"/>
+      <c r="P22" s="88"/>
+      <c r="Q22" s="88"/>
+    </row>
+    <row r="23" s="4" customFormat="1" ht="11.4" customHeight="1" spans="1:17">
+      <c r="B23" s="91" t="s">
+        <v>272</v>
+      </c>
+      <c r="C23" s="82"/>
+      <c r="D23" s="81" t="s">
+        <v>70</v>
+      </c>
+      <c r="E23" s="81" t="s">
+        <v>273</v>
+      </c>
+      <c r="F23" s="85"/>
+      <c r="G23" s="85"/>
+      <c r="H23" s="85"/>
+      <c r="I23" s="85"/>
+      <c r="J23" s="85"/>
+      <c r="L23" s="87"/>
+      <c r="M23" s="81"/>
+      <c r="N23" s="87"/>
+      <c r="O23" s="87"/>
+      <c r="P23" s="92"/>
+      <c r="Q23" s="93"/>
+    </row>
+    <row r="24" s="4" customFormat="1" ht="10.8" customHeight="1" spans="1:17">
+      <c r="B24" s="91" t="s">
+        <v>84</v>
+      </c>
+      <c r="C24" s="82"/>
+      <c r="D24" s="81" t="s">
+        <v>77</v>
+      </c>
+      <c r="E24" s="81" t="s">
+        <v>86</v>
+      </c>
+      <c r="F24" s="85"/>
+      <c r="G24" s="85"/>
+      <c r="H24" s="85"/>
+      <c r="I24" s="85"/>
+      <c r="J24" s="85"/>
+      <c r="L24" s="96"/>
+      <c r="M24" s="97"/>
+      <c r="N24" s="97"/>
+      <c r="O24" s="97"/>
+      <c r="P24" s="92"/>
+      <c r="Q24" s="93"/>
+    </row>
+    <row r="25" s="4" customFormat="1" ht="10.8" customHeight="1" spans="1:17">
+      <c r="B25" s="73" t="s">
+        <v>99</v>
+      </c>
+      <c r="C25" s="12"/>
+      <c r="D25" s="12"/>
+      <c r="E25" s="12"/>
+      <c r="F25" s="12"/>
+      <c r="G25" s="12"/>
+      <c r="H25" s="12"/>
+      <c r="I25" s="12"/>
+      <c r="J25" s="13"/>
+      <c r="L25" s="38" t="s">
+        <v>100</v>
+      </c>
+      <c r="M25" s="39"/>
+      <c r="N25" s="39"/>
+      <c r="O25" s="39"/>
+      <c r="P25" s="39"/>
+      <c r="Q25" s="40"/>
+    </row>
+    <row r="26" ht="13.95" customHeight="1" spans="1:17">
+      <c r="B26" s="98" t="s">
+        <v>7</v>
+      </c>
+      <c r="C26" s="98" t="s">
+        <v>101</v>
+      </c>
+      <c r="D26" s="98" t="s">
+        <v>45</v>
+      </c>
+      <c r="E26" s="12"/>
+      <c r="F26" s="12"/>
+      <c r="G26" s="12"/>
+      <c r="H26" s="12"/>
+      <c r="I26" s="12"/>
+      <c r="J26" s="13"/>
+      <c r="L26" s="99" t="s">
+        <v>102</v>
+      </c>
+      <c r="M26" s="100" t="s">
+        <v>103</v>
+      </c>
+      <c r="N26" s="23" t="s">
+        <v>104</v>
+      </c>
+      <c r="O26" s="23" t="s">
+        <v>105</v>
+      </c>
+      <c r="P26" s="42" t="s">
+        <v>106</v>
+      </c>
+      <c r="Q26" s="40"/>
+    </row>
+    <row r="27" ht="13.95" customHeight="1" spans="1:17">
+      <c r="B27" s="101"/>
+      <c r="C27" s="102"/>
+      <c r="D27" s="86"/>
+      <c r="E27" s="12"/>
+      <c r="F27" s="12"/>
+      <c r="G27" s="12"/>
+      <c r="H27" s="12"/>
+      <c r="I27" s="12"/>
+      <c r="J27" s="13"/>
+      <c r="L27" s="35"/>
+      <c r="M27" s="36"/>
+      <c r="N27" s="46"/>
+      <c r="O27" s="46"/>
+      <c r="P27" s="45"/>
+      <c r="Q27" s="40"/>
+    </row>
+    <row r="28" ht="13.95" customHeight="1" spans="1:17">
+      <c r="L28" s="35"/>
+      <c r="M28" s="36"/>
+      <c r="N28" s="46"/>
+      <c r="O28" s="46"/>
+      <c r="P28" s="45"/>
+      <c r="Q28" s="40"/>
+    </row>
+    <row r="29" ht="13.95" customHeight="1" spans="1:17">
+      <c r="L29" s="35"/>
+      <c r="M29" s="36"/>
+      <c r="N29" s="46"/>
+      <c r="O29" s="46"/>
+      <c r="P29" s="45"/>
+      <c r="Q29" s="40"/>
+    </row>
+    <row r="30" ht="13.95" customHeight="1" spans="1:17">
+      <c r="L30" s="35"/>
+      <c r="M30" s="36"/>
+      <c r="N30" s="46"/>
+      <c r="O30" s="46"/>
+      <c r="P30" s="103"/>
+      <c r="Q30" s="40"/>
+    </row>
+    <row r="31" ht="13.95" customHeight="1" spans="1:17">
+      <c r="L31" s="35"/>
+      <c r="M31" s="36"/>
+      <c r="N31" s="46"/>
+      <c r="O31" s="46"/>
+      <c r="P31" s="103"/>
+      <c r="Q31" s="40"/>
+    </row>
+    <row r="32" ht="13.95" customHeight="1" spans="1:17">
+      <c r="L32" s="104"/>
+      <c r="M32" s="93"/>
+      <c r="N32" s="93"/>
+      <c r="O32" s="93"/>
+      <c r="P32" s="103"/>
+      <c r="Q32" s="40"/>
+    </row>
+    <row r="33" ht="13.95" customHeight="1" spans="12:17">
+      <c r="L33" s="104"/>
+      <c r="M33" s="93"/>
+      <c r="N33" s="93"/>
+      <c r="O33" s="93"/>
+      <c r="P33" s="103"/>
+      <c r="Q33" s="40"/>
+    </row>
+    <row r="34" ht="56" customHeight="1" spans="12:17">
+      <c r="L34" s="104"/>
+      <c r="M34" s="93"/>
+      <c r="N34" s="93"/>
+      <c r="O34" s="93"/>
+      <c r="P34" s="103"/>
+      <c r="Q34" s="40"/>
+    </row>
+    <row r="35" ht="13.95" customHeight="1" spans="12:17">
+      <c r="L35" s="104"/>
+      <c r="M35" s="93"/>
+      <c r="N35" s="93"/>
+      <c r="O35" s="93"/>
+      <c r="P35" s="103"/>
+      <c r="Q35" s="40"/>
+    </row>
+    <row r="36" ht="13.95" customHeight="1" spans="12:17">
+      <c r="L36" s="66"/>
+      <c r="M36" s="67"/>
+      <c r="N36" s="68"/>
+      <c r="O36" s="93"/>
+      <c r="P36" s="69"/>
+      <c r="Q36" s="40"/>
+    </row>
+    <row r="37" ht="13.95" customHeight="1" spans="12:17">
+      <c r="L37" s="105" t="s">
+        <v>119</v>
+      </c>
+      <c r="M37" s="39"/>
+      <c r="N37" s="39"/>
+      <c r="O37" s="39"/>
+      <c r="P37" s="39"/>
+      <c r="Q37" s="40"/>
+    </row>
+    <row r="38" ht="13.95" customHeight="1" spans="12:17">
+      <c r="L38" s="106"/>
+      <c r="M38" s="39"/>
+      <c r="N38" s="39"/>
+      <c r="O38" s="39"/>
+      <c r="P38" s="39"/>
+      <c r="Q38" s="40"/>
+    </row>
+    <row r="39" ht="13.95" customHeight="1"/>
+    <row r="40" ht="13.95" customHeight="1"/>
+    <row r="41" ht="13.95" customHeight="1"/>
+    <row r="42" ht="13.95" customHeight="1"/>
+    <row r="43" ht="13.95" customHeight="1"/>
+    <row r="44" ht="13.95" customHeight="1"/>
+    <row r="45" ht="13.95" customHeight="1"/>
+    <row r="46" ht="13.95" customHeight="1"/>
+    <row r="47" ht="13.95" customHeight="1"/>
+    <row r="48" ht="13.95" customHeight="1"/>
+    <row r="49" ht="13.95" customHeight="1"/>
+    <row r="50" ht="13.95" customHeight="1"/>
+    <row r="51" ht="13.95" customHeight="1"/>
+    <row r="52" ht="13.95" customHeight="1"/>
+    <row r="53" ht="13.95" customHeight="1"/>
+    <row r="54" ht="13.95" customHeight="1"/>
+    <row r="55" ht="13.95" customHeight="1"/>
+    <row r="56" ht="13.95" customHeight="1"/>
+    <row r="57" ht="13.95" customHeight="1"/>
+    <row r="58" ht="13.95" customHeight="1"/>
+    <row r="59" ht="13.95" customHeight="1"/>
+    <row r="60" ht="13.95" customHeight="1"/>
+    <row r="61" ht="13.95" customHeight="1"/>
+    <row r="62" ht="13.95" customHeight="1"/>
+    <row r="63" ht="13.95" customHeight="1"/>
+    <row r="64" ht="13.95" customHeight="1"/>
+    <row r="65" ht="13.95" customHeight="1"/>
+    <row r="66" ht="13.95" customHeight="1"/>
+    <row r="67" ht="13.95" customHeight="1"/>
+    <row r="68" ht="13.95" customHeight="1"/>
+    <row r="69" ht="13.95" customHeight="1"/>
+    <row r="70" ht="13.95" customHeight="1"/>
+    <row r="71" ht="13.95" customHeight="1"/>
+    <row r="72" ht="13.95" customHeight="1"/>
+    <row r="73" ht="13.95" customHeight="1"/>
+    <row r="74" ht="13.95" customHeight="1"/>
+    <row r="75" ht="13.95" customHeight="1"/>
+    <row r="76" ht="13.95" customHeight="1"/>
+    <row r="77" ht="13.95" customHeight="1"/>
+    <row r="78" ht="13.95" customHeight="1"/>
+    <row r="79" ht="13.95" customHeight="1"/>
+    <row r="80" ht="13.95" customHeight="1"/>
+    <row r="81" ht="13.95" customHeight="1"/>
+    <row r="82" ht="13.95" customHeight="1"/>
+    <row r="83" ht="13.95" customHeight="1"/>
+  </sheetData>
+  <mergeCells count="23">
+    <mergeCell ref="B1:J1"/>
+    <mergeCell ref="C2:E2"/>
+    <mergeCell ref="F2:J2"/>
+    <mergeCell ref="B3:J3"/>
+    <mergeCell ref="B4:J4"/>
+    <mergeCell ref="L4:Q4"/>
+    <mergeCell ref="F5:G5"/>
+    <mergeCell ref="F19:G19"/>
+    <mergeCell ref="F20:G20"/>
+    <mergeCell ref="L21:Q21"/>
+    <mergeCell ref="P22:Q22"/>
+    <mergeCell ref="P23:Q23"/>
+    <mergeCell ref="P24:Q24"/>
+    <mergeCell ref="P25:Q25"/>
+    <mergeCell ref="P26:Q26"/>
+    <mergeCell ref="P27:Q27"/>
+    <mergeCell ref="P28:Q28"/>
+    <mergeCell ref="P29:Q29"/>
+    <mergeCell ref="P30:Q30"/>
+    <mergeCell ref="P31:Q31"/>
+    <mergeCell ref="P32:Q32"/>
+    <mergeCell ref="L33:Q33"/>
+    <mergeCell ref="L34:Q34"/>
+  </mergeCells>
+  <dataValidations count="1">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="C20">
+      <formula1>#REF!</formula1>
+    </dataValidation>
+  </dataValidations>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <headerFooter/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
+  <sheetPr/>
   <dimension ref="A1:Q84"/>
   <sheetFormatPr defaultColWidth="8.23148148148148" defaultRowHeight="14.4"/>
   <cols>
@@ -6958,12 +7780,12 @@
         <v>16</v>
       </c>
       <c r="C2" s="74" t="s">
-        <v>274</v>
+        <v>276</v>
       </c>
       <c r="D2" s="12"/>
       <c r="E2" s="12"/>
       <c r="F2" s="75" t="s">
-        <v>275</v>
+        <v>277</v>
       </c>
       <c r="G2" s="12"/>
       <c r="H2" s="12"/>
@@ -7129,7 +7951,7 @@
         <v>80</v>
       </c>
       <c r="E9" s="81" t="s">
-        <v>276</v>
+        <v>278</v>
       </c>
       <c r="F9" s="83"/>
       <c r="G9" s="83"/>
@@ -7170,14 +7992,14 @@
     <row r="11" s="6" customFormat="1" ht="13.95" customHeight="1" spans="1:17">
       <c r="A11" s="80"/>
       <c r="B11" s="89" t="s">
-        <v>277</v>
+        <v>279</v>
       </c>
       <c r="C11" s="82"/>
       <c r="D11" s="81" t="s">
         <v>80</v>
       </c>
       <c r="E11" s="81" t="s">
-        <v>278</v>
+        <v>280</v>
       </c>
       <c r="F11" s="83"/>
       <c r="G11" s="83"/>
@@ -7618,7 +8440,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
   <dimension ref="A1:Y120"/>
@@ -7645,22 +8467,22 @@
   <sheetData>
     <row r="1" ht="35" customHeight="1" spans="1:25">
       <c r="A1" s="7" t="s">
-        <v>279</v>
+        <v>281</v>
       </c>
       <c r="B1" s="8" t="s">
-        <v>280</v>
+        <v>282</v>
       </c>
       <c r="C1" s="9" t="s">
-        <v>281</v>
+        <v>283</v>
       </c>
       <c r="D1" s="9" t="s">
-        <v>282</v>
+        <v>284</v>
       </c>
       <c r="E1" s="10"/>
     </row>
     <row r="2" ht="56" customHeight="1" spans="1:25">
       <c r="A2" s="11" t="s">
-        <v>283</v>
+        <v>285</v>
       </c>
       <c r="B2" s="12"/>
       <c r="C2" s="12"/>
@@ -7669,7 +8491,7 @@
     </row>
     <row r="3" ht="23" customHeight="1" spans="1:25">
       <c r="A3" s="14" t="s">
-        <v>284</v>
+        <v>286</v>
       </c>
       <c r="B3" s="15">
         <v>1</v>
@@ -7700,66 +8522,66 @@
     </row>
     <row r="4" s="3" customFormat="1" ht="34" customHeight="1" spans="1:25">
       <c r="A4" s="17" t="s">
-        <v>285</v>
+        <v>287</v>
       </c>
       <c r="B4" s="12"/>
       <c r="C4" s="12"/>
       <c r="D4" s="13"/>
       <c r="E4" s="18"/>
       <c r="F4" s="19" t="s">
-        <v>286</v>
+        <v>288</v>
       </c>
       <c r="G4" s="19" t="s">
-        <v>287</v>
+        <v>289</v>
       </c>
       <c r="H4" s="13"/>
       <c r="I4" s="19" t="s">
-        <v>288</v>
+        <v>290</v>
       </c>
       <c r="J4" s="19" t="s">
-        <v>289</v>
+        <v>291</v>
       </c>
       <c r="K4" s="13"/>
       <c r="L4" s="18"/>
       <c r="M4" s="19" t="s">
-        <v>290</v>
+        <v>292</v>
       </c>
       <c r="N4" s="19" t="s">
-        <v>291</v>
+        <v>293</v>
       </c>
       <c r="O4" s="13"/>
       <c r="P4" s="19" t="s">
-        <v>288</v>
+        <v>290</v>
       </c>
       <c r="Q4" s="19" t="s">
-        <v>289</v>
+        <v>291</v>
       </c>
       <c r="R4" s="13"/>
       <c r="S4" s="18"/>
       <c r="T4" s="19" t="s">
-        <v>292</v>
+        <v>294</v>
       </c>
       <c r="U4" s="19" t="s">
-        <v>293</v>
+        <v>295</v>
       </c>
       <c r="V4" s="13"/>
       <c r="W4" s="19" t="s">
-        <v>288</v>
+        <v>290</v>
       </c>
       <c r="X4" s="19" t="s">
-        <v>289</v>
+        <v>291</v>
       </c>
       <c r="Y4" s="13"/>
     </row>
     <row r="5" s="4" customFormat="1" ht="16.95" customHeight="1" spans="1:25">
       <c r="A5" s="20" t="s">
-        <v>294</v>
+        <v>296</v>
       </c>
       <c r="B5" s="20" t="s">
-        <v>295</v>
+        <v>297</v>
       </c>
       <c r="C5" s="20" t="s">
-        <v>296</v>
+        <v>298</v>
       </c>
       <c r="D5" s="20" t="s">
         <v>186</v>
@@ -7769,7 +8591,7 @@
         <v>40</v>
       </c>
       <c r="G5" s="23" t="s">
-        <v>297</v>
+        <v>299</v>
       </c>
       <c r="H5" s="23" t="s">
         <v>42</v>
@@ -7788,7 +8610,7 @@
         <v>40</v>
       </c>
       <c r="N5" s="23" t="s">
-        <v>297</v>
+        <v>299</v>
       </c>
       <c r="O5" s="23" t="s">
         <v>42</v>
@@ -7807,7 +8629,7 @@
         <v>40</v>
       </c>
       <c r="U5" s="23" t="s">
-        <v>297</v>
+        <v>299</v>
       </c>
       <c r="V5" s="23" t="s">
         <v>42</v>
@@ -7824,7 +8646,7 @@
     </row>
     <row r="6" s="4" customFormat="1" ht="16.95" customHeight="1" spans="1:25">
       <c r="A6" s="25" t="s">
-        <v>298</v>
+        <v>300</v>
       </c>
       <c r="B6" s="26" t="s">
         <v>84</v>
@@ -7835,7 +8657,7 @@
       <c r="D6" s="27"/>
       <c r="E6" s="21"/>
       <c r="F6" s="28" t="s">
-        <v>299</v>
+        <v>301</v>
       </c>
       <c r="G6" s="28" t="s">
         <v>109</v>
@@ -7850,7 +8672,7 @@
       <c r="K6" s="28"/>
       <c r="L6" s="21"/>
       <c r="M6" s="28" t="s">
-        <v>300</v>
+        <v>302</v>
       </c>
       <c r="N6" s="28" t="s">
         <v>109</v>
@@ -7865,7 +8687,7 @@
       <c r="R6" s="28"/>
       <c r="S6" s="21"/>
       <c r="T6" s="28" t="s">
-        <v>301</v>
+        <v>303</v>
       </c>
       <c r="U6" s="28" t="s">
         <v>109</v>
@@ -7881,7 +8703,7 @@
     </row>
     <row r="7" s="5" customFormat="1" ht="13.95" customHeight="1" spans="1:25">
       <c r="A7" s="25" t="s">
-        <v>298</v>
+        <v>300</v>
       </c>
       <c r="B7" s="26" t="s">
         <v>61</v>
@@ -7892,7 +8714,7 @@
       <c r="D7" s="27"/>
       <c r="E7" s="31"/>
       <c r="F7" s="28" t="s">
-        <v>299</v>
+        <v>301</v>
       </c>
       <c r="G7" s="28" t="s">
         <v>109</v>
@@ -7907,7 +8729,7 @@
       <c r="K7" s="28"/>
       <c r="L7" s="31"/>
       <c r="M7" s="28" t="s">
-        <v>300</v>
+        <v>302</v>
       </c>
       <c r="N7" s="28" t="s">
         <v>109</v>
@@ -7922,7 +8744,7 @@
       <c r="R7" s="28"/>
       <c r="S7" s="31"/>
       <c r="T7" s="28" t="s">
-        <v>301</v>
+        <v>303</v>
       </c>
       <c r="U7" s="28" t="s">
         <v>109</v>
@@ -7938,7 +8760,7 @@
     </row>
     <row r="8" s="5" customFormat="1" ht="13.95" customHeight="1" spans="1:25">
       <c r="A8" s="25" t="s">
-        <v>298</v>
+        <v>300</v>
       </c>
       <c r="B8" s="26" t="s">
         <v>65</v>
@@ -7949,7 +8771,7 @@
       <c r="D8" s="27"/>
       <c r="E8" s="31"/>
       <c r="F8" s="28" t="s">
-        <v>302</v>
+        <v>304</v>
       </c>
       <c r="G8" s="28" t="s">
         <v>112</v>
@@ -7964,7 +8786,7 @@
       <c r="K8" s="28"/>
       <c r="L8" s="31"/>
       <c r="M8" s="28" t="s">
-        <v>302</v>
+        <v>304</v>
       </c>
       <c r="N8" s="28" t="s">
         <v>112</v>
@@ -7979,7 +8801,7 @@
       <c r="R8" s="28"/>
       <c r="S8" s="31"/>
       <c r="T8" s="28" t="s">
-        <v>302</v>
+        <v>304</v>
       </c>
       <c r="U8" s="28" t="s">
         <v>112</v>
@@ -7995,18 +8817,18 @@
     </row>
     <row r="9" s="5" customFormat="1" ht="13.95" customHeight="1" spans="1:25">
       <c r="A9" s="25" t="s">
-        <v>298</v>
+        <v>300</v>
       </c>
       <c r="B9" s="26" t="s">
         <v>172</v>
       </c>
       <c r="C9" s="26" t="s">
-        <v>303</v>
+        <v>305</v>
       </c>
       <c r="D9" s="26"/>
       <c r="E9" s="31"/>
       <c r="F9" s="28" t="s">
-        <v>302</v>
+        <v>304</v>
       </c>
       <c r="G9" s="28" t="s">
         <v>112</v>
@@ -8015,13 +8837,13 @@
         <v>172</v>
       </c>
       <c r="I9" s="30" t="s">
-        <v>303</v>
+        <v>305</v>
       </c>
       <c r="J9" s="32"/>
       <c r="K9" s="28"/>
       <c r="L9" s="31"/>
       <c r="M9" s="28" t="s">
-        <v>302</v>
+        <v>304</v>
       </c>
       <c r="N9" s="28" t="s">
         <v>112</v>
@@ -8030,13 +8852,13 @@
         <v>172</v>
       </c>
       <c r="P9" s="30" t="s">
-        <v>303</v>
+        <v>305</v>
       </c>
       <c r="Q9" s="32"/>
       <c r="R9" s="28"/>
       <c r="S9" s="31"/>
       <c r="T9" s="28" t="s">
-        <v>302</v>
+        <v>304</v>
       </c>
       <c r="U9" s="28" t="s">
         <v>112</v>
@@ -8045,25 +8867,25 @@
         <v>172</v>
       </c>
       <c r="W9" s="30" t="s">
-        <v>303</v>
+        <v>305</v>
       </c>
       <c r="X9" s="32"/>
       <c r="Y9" s="28"/>
     </row>
     <row r="10" s="6" customFormat="1" ht="13.95" customHeight="1" spans="1:25">
       <c r="A10" s="25" t="s">
-        <v>298</v>
+        <v>300</v>
       </c>
       <c r="B10" s="26" t="s">
         <v>92</v>
       </c>
       <c r="C10" s="26" t="s">
-        <v>304</v>
+        <v>306</v>
       </c>
       <c r="D10" s="26"/>
       <c r="E10" s="33"/>
       <c r="F10" s="28" t="s">
-        <v>302</v>
+        <v>304</v>
       </c>
       <c r="G10" s="28" t="s">
         <v>112</v>
@@ -8072,13 +8894,13 @@
         <v>92</v>
       </c>
       <c r="I10" s="30" t="s">
-        <v>304</v>
+        <v>306</v>
       </c>
       <c r="J10" s="32"/>
       <c r="K10" s="28"/>
       <c r="L10" s="33"/>
       <c r="M10" s="28" t="s">
-        <v>302</v>
+        <v>304</v>
       </c>
       <c r="N10" s="28" t="s">
         <v>112</v>
@@ -8087,13 +8909,13 @@
         <v>92</v>
       </c>
       <c r="P10" s="30" t="s">
-        <v>304</v>
+        <v>306</v>
       </c>
       <c r="Q10" s="32"/>
       <c r="R10" s="28"/>
       <c r="S10" s="33"/>
       <c r="T10" s="28" t="s">
-        <v>302</v>
+        <v>304</v>
       </c>
       <c r="U10" s="28" t="s">
         <v>112</v>
@@ -8102,25 +8924,25 @@
         <v>92</v>
       </c>
       <c r="W10" s="30" t="s">
-        <v>304</v>
+        <v>306</v>
       </c>
       <c r="X10" s="32"/>
       <c r="Y10" s="28"/>
     </row>
     <row r="11" s="6" customFormat="1" ht="13.95" customHeight="1" spans="1:25">
       <c r="A11" s="25" t="s">
-        <v>298</v>
+        <v>300</v>
       </c>
       <c r="B11" s="26" t="s">
-        <v>305</v>
+        <v>307</v>
       </c>
       <c r="C11" s="34" t="s">
-        <v>306</v>
+        <v>308</v>
       </c>
       <c r="D11" s="34"/>
       <c r="E11" s="33"/>
       <c r="F11" s="28" t="s">
-        <v>299</v>
+        <v>301</v>
       </c>
       <c r="G11" s="28" t="s">
         <v>109</v>
@@ -8135,7 +8957,7 @@
       <c r="K11" s="32"/>
       <c r="L11" s="33"/>
       <c r="M11" s="28" t="s">
-        <v>300</v>
+        <v>302</v>
       </c>
       <c r="N11" s="28" t="s">
         <v>109</v>
@@ -8144,55 +8966,55 @@
         <v>215</v>
       </c>
       <c r="P11" s="30" t="s">
-        <v>307</v>
+        <v>309</v>
       </c>
       <c r="Q11" s="32"/>
       <c r="R11" s="32"/>
       <c r="S11" s="33"/>
       <c r="T11" s="28" t="s">
-        <v>301</v>
+        <v>303</v>
       </c>
       <c r="U11" s="28" t="s">
         <v>109</v>
       </c>
       <c r="V11" s="29" t="s">
-        <v>308</v>
+        <v>310</v>
       </c>
       <c r="W11" s="30" t="s">
-        <v>307</v>
+        <v>309</v>
       </c>
       <c r="X11" s="32"/>
       <c r="Y11" s="32"/>
     </row>
     <row r="12" s="6" customFormat="1" ht="13.95" customHeight="1" spans="1:25">
       <c r="A12" s="25" t="s">
-        <v>298</v>
+        <v>300</v>
       </c>
       <c r="B12" s="26" t="s">
-        <v>309</v>
+        <v>311</v>
       </c>
       <c r="C12" s="27" t="s">
-        <v>310</v>
+        <v>312</v>
       </c>
       <c r="D12" s="27"/>
       <c r="E12" s="33"/>
       <c r="F12" s="28" t="s">
-        <v>299</v>
+        <v>301</v>
       </c>
       <c r="G12" s="28" t="s">
         <v>109</v>
       </c>
       <c r="H12" s="35" t="s">
-        <v>311</v>
+        <v>313</v>
       </c>
       <c r="I12" s="36" t="s">
-        <v>312</v>
+        <v>314</v>
       </c>
       <c r="J12" s="28"/>
       <c r="K12" s="28"/>
       <c r="L12" s="33"/>
       <c r="M12" s="28" t="s">
-        <v>300</v>
+        <v>302</v>
       </c>
       <c r="N12" s="28" t="s">
         <v>109</v>
@@ -8201,55 +9023,55 @@
         <v>211</v>
       </c>
       <c r="P12" s="30" t="s">
-        <v>313</v>
+        <v>315</v>
       </c>
       <c r="Q12" s="28"/>
       <c r="R12" s="28"/>
       <c r="S12" s="33"/>
       <c r="T12" s="28" t="s">
-        <v>301</v>
+        <v>303</v>
       </c>
       <c r="U12" s="28" t="s">
         <v>109</v>
       </c>
       <c r="V12" s="29" t="s">
-        <v>314</v>
+        <v>316</v>
       </c>
       <c r="W12" s="30" t="s">
-        <v>315</v>
+        <v>317</v>
       </c>
       <c r="X12" s="28"/>
       <c r="Y12" s="28"/>
     </row>
     <row r="13" s="6" customFormat="1" ht="13.95" customHeight="1" spans="1:25">
       <c r="A13" s="25" t="s">
-        <v>298</v>
+        <v>300</v>
       </c>
       <c r="B13" s="26" t="s">
-        <v>316</v>
+        <v>318</v>
       </c>
       <c r="C13" s="27" t="s">
-        <v>317</v>
+        <v>319</v>
       </c>
       <c r="D13" s="27"/>
       <c r="E13" s="33"/>
       <c r="F13" s="28" t="s">
-        <v>299</v>
+        <v>301</v>
       </c>
       <c r="G13" s="28" t="s">
         <v>109</v>
       </c>
       <c r="H13" s="35" t="s">
-        <v>318</v>
+        <v>320</v>
       </c>
       <c r="I13" s="36" t="s">
-        <v>319</v>
+        <v>321</v>
       </c>
       <c r="J13" s="28"/>
       <c r="K13" s="28"/>
       <c r="L13" s="33"/>
       <c r="M13" s="28" t="s">
-        <v>300</v>
+        <v>302</v>
       </c>
       <c r="N13" s="28" t="s">
         <v>109</v>
@@ -8264,16 +9086,16 @@
       <c r="R13" s="28"/>
       <c r="S13" s="33"/>
       <c r="T13" s="28" t="s">
-        <v>301</v>
+        <v>303</v>
       </c>
       <c r="U13" s="28" t="s">
         <v>109</v>
       </c>
       <c r="V13" s="29" t="s">
-        <v>320</v>
+        <v>322</v>
       </c>
       <c r="W13" s="30" t="s">
-        <v>321</v>
+        <v>323</v>
       </c>
       <c r="X13" s="28"/>
       <c r="Y13" s="28"/>
@@ -8408,10 +9230,10 @@
       <c r="D17" s="13"/>
       <c r="E17" s="21"/>
       <c r="F17" s="28" t="s">
-        <v>299</v>
+        <v>301</v>
       </c>
       <c r="G17" s="28" t="s">
-        <v>322</v>
+        <v>324</v>
       </c>
       <c r="H17" s="29" t="s">
         <v>109</v>
@@ -8421,10 +9243,10 @@
       <c r="K17" s="40"/>
       <c r="L17" s="21"/>
       <c r="M17" s="28" t="s">
-        <v>300</v>
+        <v>302</v>
       </c>
       <c r="N17" s="28" t="s">
-        <v>323</v>
+        <v>325</v>
       </c>
       <c r="O17" s="29" t="s">
         <v>109</v>
@@ -8434,10 +9256,10 @@
       <c r="R17" s="40"/>
       <c r="S17" s="21"/>
       <c r="T17" s="28" t="s">
-        <v>301</v>
+        <v>303</v>
       </c>
       <c r="U17" s="28" t="s">
-        <v>324</v>
+        <v>326</v>
       </c>
       <c r="V17" s="29" t="s">
         <v>109</v>
@@ -8453,53 +9275,53 @@
       <c r="D18" s="21"/>
       <c r="E18" s="21"/>
       <c r="F18" s="28" t="s">
-        <v>302</v>
+        <v>304</v>
       </c>
       <c r="G18" s="28" t="s">
-        <v>325</v>
+        <v>327</v>
       </c>
       <c r="H18" s="29" t="s">
         <v>112</v>
       </c>
       <c r="I18" s="30" t="s">
-        <v>326</v>
+        <v>328</v>
       </c>
       <c r="J18" s="45" t="s">
-        <v>327</v>
+        <v>329</v>
       </c>
       <c r="K18" s="40"/>
       <c r="L18" s="21"/>
       <c r="M18" s="28" t="s">
-        <v>302</v>
+        <v>304</v>
       </c>
       <c r="N18" s="28" t="s">
-        <v>325</v>
+        <v>327</v>
       </c>
       <c r="O18" s="29" t="s">
         <v>112</v>
       </c>
       <c r="P18" s="30" t="s">
-        <v>326</v>
+        <v>328</v>
       </c>
       <c r="Q18" s="45" t="s">
-        <v>327</v>
+        <v>329</v>
       </c>
       <c r="R18" s="40"/>
       <c r="S18" s="21"/>
       <c r="T18" s="28" t="s">
-        <v>302</v>
+        <v>304</v>
       </c>
       <c r="U18" s="28" t="s">
-        <v>325</v>
+        <v>327</v>
       </c>
       <c r="V18" s="29" t="s">
         <v>112</v>
       </c>
       <c r="W18" s="30" t="s">
-        <v>326</v>
+        <v>328</v>
       </c>
       <c r="X18" s="45" t="s">
-        <v>327</v>
+        <v>329</v>
       </c>
       <c r="Y18" s="40"/>
     </row>
@@ -8570,7 +9392,7 @@
       <c r="D21" s="16"/>
       <c r="E21" s="16"/>
       <c r="F21" s="47" t="s">
-        <v>328</v>
+        <v>330</v>
       </c>
       <c r="G21" s="39"/>
       <c r="H21" s="39"/>
@@ -8579,7 +9401,7 @@
       <c r="K21" s="40"/>
       <c r="L21" s="16"/>
       <c r="M21" s="47" t="s">
-        <v>329</v>
+        <v>331</v>
       </c>
       <c r="N21" s="39"/>
       <c r="O21" s="39"/>
@@ -8588,7 +9410,7 @@
       <c r="R21" s="40"/>
       <c r="S21" s="16"/>
       <c r="T21" s="47" t="s">
-        <v>330</v>
+        <v>332</v>
       </c>
       <c r="U21" s="39"/>
       <c r="V21" s="39"/>
@@ -8599,7 +9421,7 @@
     <row r="22" ht="13.95" customHeight="1"/>
     <row r="23" ht="13.95" customHeight="1" spans="1:25">
       <c r="A23" s="14" t="s">
-        <v>284</v>
+        <v>286</v>
       </c>
       <c r="B23" s="15">
         <v>2</v>
@@ -8616,24 +9438,24 @@
     </row>
     <row r="24" ht="36" customHeight="1" spans="1:25">
       <c r="A24" s="17" t="s">
-        <v>285</v>
+        <v>287</v>
       </c>
       <c r="B24" s="12"/>
       <c r="C24" s="12"/>
       <c r="D24" s="13"/>
       <c r="E24" s="18"/>
       <c r="F24" s="19" t="s">
-        <v>286</v>
+        <v>288</v>
       </c>
       <c r="G24" s="19" t="s">
-        <v>331</v>
+        <v>333</v>
       </c>
       <c r="H24" s="13"/>
       <c r="I24" s="19" t="s">
-        <v>288</v>
+        <v>290</v>
       </c>
       <c r="J24" s="19" t="s">
-        <v>289</v>
+        <v>291</v>
       </c>
       <c r="K24" s="13"/>
       <c r="M24" s="48"/>
@@ -8643,13 +9465,13 @@
     </row>
     <row r="25" ht="29" customHeight="1" spans="1:25">
       <c r="A25" s="20" t="s">
-        <v>294</v>
+        <v>296</v>
       </c>
       <c r="B25" s="20" t="s">
-        <v>295</v>
+        <v>297</v>
       </c>
       <c r="C25" s="20" t="s">
-        <v>296</v>
+        <v>298</v>
       </c>
       <c r="D25" s="20" t="s">
         <v>186</v>
@@ -8659,7 +9481,7 @@
         <v>40</v>
       </c>
       <c r="G25" s="23" t="s">
-        <v>297</v>
+        <v>299</v>
       </c>
       <c r="H25" s="23" t="s">
         <v>42</v>
@@ -8682,7 +9504,7 @@
     </row>
     <row r="26" ht="13.95" customHeight="1" spans="1:25">
       <c r="A26" s="25" t="s">
-        <v>332</v>
+        <v>334</v>
       </c>
       <c r="B26" s="52" t="s">
         <v>84</v>
@@ -8697,7 +9519,7 @@
       <c r="H26" s="29"/>
       <c r="I26" s="30"/>
       <c r="J26" s="178" t="s">
-        <v>333</v>
+        <v>335</v>
       </c>
       <c r="K26" s="28"/>
       <c r="M26" s="53"/>
@@ -8709,13 +9531,13 @@
     </row>
     <row r="27" ht="13.95" customHeight="1" spans="1:25">
       <c r="A27" s="25" t="s">
-        <v>332</v>
+        <v>334</v>
       </c>
       <c r="B27" s="52" t="s">
-        <v>334</v>
+        <v>336</v>
       </c>
       <c r="C27" s="27" t="s">
-        <v>335</v>
+        <v>337</v>
       </c>
       <c r="D27" s="27"/>
       <c r="E27" s="21"/>
@@ -8723,10 +9545,10 @@
       <c r="G27" s="28"/>
       <c r="H27" s="29"/>
       <c r="I27" s="30" t="s">
-        <v>336</v>
+        <v>338</v>
       </c>
       <c r="J27" s="28" t="s">
-        <v>337</v>
+        <v>339</v>
       </c>
       <c r="K27" s="28"/>
       <c r="M27" s="53"/>
@@ -8738,27 +9560,27 @@
     </row>
     <row r="28" ht="13.95" customHeight="1" spans="1:25">
       <c r="A28" s="25" t="s">
-        <v>332</v>
+        <v>334</v>
       </c>
       <c r="B28" s="52" t="s">
-        <v>338</v>
+        <v>340</v>
       </c>
       <c r="C28" s="27" t="s">
-        <v>339</v>
+        <v>341</v>
       </c>
       <c r="D28" s="27"/>
       <c r="E28" s="31"/>
       <c r="F28" s="28" t="s">
-        <v>340</v>
+        <v>342</v>
       </c>
       <c r="G28" s="28" t="s">
         <v>109</v>
       </c>
       <c r="H28" s="29" t="s">
-        <v>341</v>
+        <v>343</v>
       </c>
       <c r="I28" s="30" t="s">
-        <v>342</v>
+        <v>344</v>
       </c>
       <c r="J28" s="28"/>
       <c r="K28" s="28"/>
@@ -8771,16 +9593,16 @@
     </row>
     <row r="29" ht="13.95" customHeight="1" spans="1:25">
       <c r="A29" s="25" t="s">
-        <v>332</v>
+        <v>334</v>
       </c>
       <c r="B29" s="52" t="s">
-        <v>343</v>
+        <v>345</v>
       </c>
       <c r="C29" s="34" t="s">
-        <v>344</v>
+        <v>346</v>
       </c>
       <c r="D29" s="34" t="s">
-        <v>345</v>
+        <v>347</v>
       </c>
       <c r="E29" s="31"/>
       <c r="F29" s="28"/>
@@ -8788,7 +9610,7 @@
       <c r="H29" s="29"/>
       <c r="I29" s="30"/>
       <c r="J29" s="178" t="s">
-        <v>346</v>
+        <v>348</v>
       </c>
       <c r="K29" s="28"/>
       <c r="M29" s="53"/>
@@ -8800,27 +9622,27 @@
     </row>
     <row r="30" ht="13.95" customHeight="1" spans="1:25">
       <c r="A30" s="25" t="s">
-        <v>332</v>
+        <v>334</v>
       </c>
       <c r="B30" s="52" t="s">
-        <v>347</v>
+        <v>349</v>
       </c>
       <c r="C30" s="34" t="s">
-        <v>348</v>
+        <v>350</v>
       </c>
       <c r="D30" s="34"/>
       <c r="E30" s="33"/>
       <c r="F30" s="28" t="s">
-        <v>340</v>
+        <v>342</v>
       </c>
       <c r="G30" s="28" t="s">
         <v>109</v>
       </c>
       <c r="H30" s="29" t="s">
-        <v>349</v>
+        <v>351</v>
       </c>
       <c r="I30" s="30" t="s">
-        <v>348</v>
+        <v>350</v>
       </c>
       <c r="J30" s="32"/>
       <c r="K30" s="28"/>
@@ -8833,27 +9655,27 @@
     </row>
     <row r="31" ht="13.95" customHeight="1" spans="1:25">
       <c r="A31" s="25" t="s">
-        <v>332</v>
+        <v>334</v>
       </c>
       <c r="B31" s="52" t="s">
-        <v>350</v>
+        <v>352</v>
       </c>
       <c r="C31" s="34" t="s">
-        <v>351</v>
+        <v>353</v>
       </c>
       <c r="D31" s="34"/>
       <c r="E31" s="33"/>
       <c r="F31" s="28" t="s">
-        <v>340</v>
+        <v>342</v>
       </c>
       <c r="G31" s="28" t="s">
         <v>109</v>
       </c>
       <c r="H31" s="29" t="s">
-        <v>350</v>
+        <v>352</v>
       </c>
       <c r="I31" s="30" t="s">
-        <v>351</v>
+        <v>353</v>
       </c>
       <c r="J31" s="28"/>
       <c r="K31" s="28"/>
@@ -8866,18 +9688,18 @@
     </row>
     <row r="32" ht="13.95" customHeight="1" spans="1:25">
       <c r="A32" s="25" t="s">
-        <v>332</v>
+        <v>334</v>
       </c>
       <c r="B32" s="52" t="s">
         <v>172</v>
       </c>
       <c r="C32" s="34" t="s">
-        <v>303</v>
+        <v>305</v>
       </c>
       <c r="D32" s="34"/>
       <c r="E32" s="33"/>
       <c r="F32" s="28" t="s">
-        <v>340</v>
+        <v>342</v>
       </c>
       <c r="G32" s="28" t="s">
         <v>109</v>
@@ -8886,7 +9708,7 @@
         <v>172</v>
       </c>
       <c r="I32" s="30" t="s">
-        <v>303</v>
+        <v>305</v>
       </c>
       <c r="J32" s="28"/>
       <c r="K32" s="28"/>
@@ -8899,18 +9721,18 @@
     </row>
     <row r="33" ht="13.95" customHeight="1" spans="1:18">
       <c r="A33" s="25" t="s">
-        <v>332</v>
+        <v>334</v>
       </c>
       <c r="B33" s="52" t="s">
         <v>170</v>
       </c>
       <c r="C33" s="34" t="s">
-        <v>352</v>
+        <v>354</v>
       </c>
       <c r="D33" s="34"/>
       <c r="E33" s="33"/>
       <c r="F33" s="28" t="s">
-        <v>340</v>
+        <v>342</v>
       </c>
       <c r="G33" s="28" t="s">
         <v>109</v>
@@ -8919,7 +9741,7 @@
         <v>170</v>
       </c>
       <c r="I33" s="30" t="s">
-        <v>352</v>
+        <v>354</v>
       </c>
       <c r="J33" s="28"/>
       <c r="K33" s="28"/>
@@ -8932,18 +9754,18 @@
     </row>
     <row r="34" ht="13.95" customHeight="1" spans="1:18">
       <c r="A34" s="25" t="s">
-        <v>332</v>
+        <v>334</v>
       </c>
       <c r="B34" s="52" t="s">
-        <v>353</v>
+        <v>355</v>
       </c>
       <c r="C34" s="34" t="s">
-        <v>354</v>
+        <v>356</v>
       </c>
       <c r="D34" s="34"/>
       <c r="E34" s="33"/>
       <c r="F34" s="28" t="s">
-        <v>340</v>
+        <v>342</v>
       </c>
       <c r="G34" s="28" t="s">
         <v>109</v>
@@ -8965,13 +9787,13 @@
     </row>
     <row r="35" ht="13.95" customHeight="1" spans="1:18">
       <c r="A35" s="25" t="s">
-        <v>332</v>
+        <v>334</v>
       </c>
       <c r="B35" s="52" t="s">
-        <v>355</v>
+        <v>357</v>
       </c>
       <c r="C35" s="34" t="s">
-        <v>356</v>
+        <v>358</v>
       </c>
       <c r="D35" s="34"/>
       <c r="E35" s="33"/>
@@ -8980,10 +9802,10 @@
       <c r="H35" s="29"/>
       <c r="I35" s="30"/>
       <c r="J35" s="178" t="s">
-        <v>357</v>
+        <v>359</v>
       </c>
       <c r="K35" s="28" t="s">
-        <v>358</v>
+        <v>360</v>
       </c>
       <c r="M35" s="53"/>
       <c r="N35" s="53"/>
@@ -8994,13 +9816,13 @@
     </row>
     <row r="36" ht="13.95" customHeight="1" spans="1:18">
       <c r="A36" s="25" t="s">
-        <v>332</v>
+        <v>334</v>
       </c>
       <c r="B36" s="52" t="s">
-        <v>359</v>
+        <v>361</v>
       </c>
       <c r="C36" s="34" t="s">
-        <v>360</v>
+        <v>362</v>
       </c>
       <c r="D36" s="34"/>
       <c r="E36" s="33"/>
@@ -9009,10 +9831,10 @@
       <c r="H36" s="29"/>
       <c r="I36" s="30"/>
       <c r="J36" s="178" t="s">
-        <v>361</v>
+        <v>363</v>
       </c>
       <c r="K36" s="28" t="s">
-        <v>362</v>
+        <v>364</v>
       </c>
       <c r="M36" s="53"/>
       <c r="N36" s="53"/>
@@ -9023,13 +9845,13 @@
     </row>
     <row r="37" ht="13.95" customHeight="1" spans="1:18">
       <c r="A37" s="25" t="s">
-        <v>332</v>
+        <v>334</v>
       </c>
       <c r="B37" s="52" t="s">
-        <v>363</v>
+        <v>365</v>
       </c>
       <c r="C37" s="34" t="s">
-        <v>364</v>
+        <v>366</v>
       </c>
       <c r="D37" s="34"/>
       <c r="E37" s="33"/>
@@ -9038,10 +9860,10 @@
       <c r="H37" s="29"/>
       <c r="I37" s="30"/>
       <c r="J37" s="28" t="s">
-        <v>365</v>
+        <v>367</v>
       </c>
       <c r="K37" s="28" t="s">
-        <v>366</v>
+        <v>368</v>
       </c>
       <c r="M37" s="53"/>
       <c r="N37" s="53"/>
@@ -9052,16 +9874,16 @@
     </row>
     <row r="38" ht="13.95" customHeight="1" spans="1:18">
       <c r="A38" s="25" t="s">
-        <v>332</v>
+        <v>334</v>
       </c>
       <c r="B38" s="52" t="s">
-        <v>367</v>
+        <v>369</v>
       </c>
       <c r="C38" s="34" t="s">
-        <v>368</v>
+        <v>370</v>
       </c>
       <c r="D38" s="34" t="s">
-        <v>369</v>
+        <v>371</v>
       </c>
       <c r="E38" s="33"/>
       <c r="F38" s="28"/>
@@ -9069,7 +9891,7 @@
       <c r="H38" s="29"/>
       <c r="I38" s="30"/>
       <c r="J38" s="28" t="s">
-        <v>370</v>
+        <v>372</v>
       </c>
       <c r="K38" s="28"/>
       <c r="M38" s="53"/>
@@ -9081,16 +9903,16 @@
     </row>
     <row r="39" ht="13.95" customHeight="1" spans="1:18">
       <c r="A39" s="25" t="s">
-        <v>332</v>
+        <v>334</v>
       </c>
       <c r="B39" s="52" t="s">
-        <v>371</v>
+        <v>373</v>
       </c>
       <c r="C39" s="34" t="s">
-        <v>372</v>
+        <v>374</v>
       </c>
       <c r="D39" s="34" t="s">
-        <v>373</v>
+        <v>375</v>
       </c>
       <c r="E39" s="33"/>
       <c r="F39" s="28"/>
@@ -9098,7 +9920,7 @@
       <c r="H39" s="29"/>
       <c r="I39" s="30"/>
       <c r="J39" s="28" t="s">
-        <v>374</v>
+        <v>376</v>
       </c>
       <c r="K39" s="28"/>
       <c r="M39" s="53"/>
@@ -9110,13 +9932,13 @@
     </row>
     <row r="40" ht="13.95" customHeight="1" spans="1:18">
       <c r="A40" s="25" t="s">
-        <v>332</v>
+        <v>334</v>
       </c>
       <c r="B40" s="52" t="s">
-        <v>375</v>
+        <v>377</v>
       </c>
       <c r="C40" s="34" t="s">
-        <v>376</v>
+        <v>378</v>
       </c>
       <c r="D40" s="34"/>
       <c r="E40" s="33"/>
@@ -9125,10 +9947,10 @@
       <c r="H40" s="29"/>
       <c r="I40" s="30"/>
       <c r="J40" s="178" t="s">
-        <v>357</v>
+        <v>359</v>
       </c>
       <c r="K40" s="28" t="s">
-        <v>358</v>
+        <v>360</v>
       </c>
       <c r="M40" s="53"/>
       <c r="N40" s="53"/>
@@ -9139,10 +9961,10 @@
     </row>
     <row r="41" ht="13.95" customHeight="1" spans="1:18">
       <c r="A41" s="25" t="s">
-        <v>332</v>
+        <v>334</v>
       </c>
       <c r="B41" s="52" t="s">
-        <v>377</v>
+        <v>379</v>
       </c>
       <c r="C41" s="27" t="s">
         <v>212</v>
@@ -9154,10 +9976,10 @@
       <c r="H41" s="29"/>
       <c r="I41" s="30"/>
       <c r="J41" s="178" t="s">
-        <v>378</v>
+        <v>380</v>
       </c>
       <c r="K41" s="28" t="s">
-        <v>379</v>
+        <v>381</v>
       </c>
       <c r="M41" s="53"/>
       <c r="N41" s="53"/>
@@ -9168,13 +9990,13 @@
     </row>
     <row r="42" ht="13.95" customHeight="1" spans="1:18">
       <c r="A42" s="25" t="s">
-        <v>332</v>
+        <v>334</v>
       </c>
       <c r="B42" s="52" t="s">
-        <v>380</v>
+        <v>382</v>
       </c>
       <c r="C42" s="27" t="s">
-        <v>381</v>
+        <v>383</v>
       </c>
       <c r="D42" s="27"/>
       <c r="E42" s="33"/>
@@ -9183,10 +10005,10 @@
       <c r="H42" s="29"/>
       <c r="I42" s="30"/>
       <c r="J42" s="178" t="s">
-        <v>357</v>
+        <v>359</v>
       </c>
       <c r="K42" s="28" t="s">
-        <v>358</v>
+        <v>360</v>
       </c>
       <c r="M42" s="53"/>
       <c r="N42" s="53"/>
@@ -9197,13 +10019,13 @@
     </row>
     <row r="43" ht="13.95" customHeight="1" spans="1:18">
       <c r="A43" s="25" t="s">
-        <v>332</v>
+        <v>334</v>
       </c>
       <c r="B43" s="52" t="s">
-        <v>382</v>
+        <v>384</v>
       </c>
       <c r="C43" s="27" t="s">
-        <v>383</v>
+        <v>385</v>
       </c>
       <c r="D43" s="27"/>
       <c r="E43" s="33"/>
@@ -9212,10 +10034,10 @@
       <c r="H43" s="29"/>
       <c r="I43" s="30"/>
       <c r="J43" s="178" t="s">
-        <v>357</v>
+        <v>359</v>
       </c>
       <c r="K43" s="28" t="s">
-        <v>358</v>
+        <v>360</v>
       </c>
       <c r="M43" s="53"/>
       <c r="N43" s="53"/>
@@ -9226,13 +10048,13 @@
     </row>
     <row r="44" ht="13.95" customHeight="1" spans="1:18">
       <c r="A44" s="25" t="s">
-        <v>332</v>
+        <v>334</v>
       </c>
       <c r="B44" s="52" t="s">
-        <v>384</v>
+        <v>386</v>
       </c>
       <c r="C44" s="27" t="s">
-        <v>385</v>
+        <v>387</v>
       </c>
       <c r="D44" s="27"/>
       <c r="E44" s="33"/>
@@ -9241,10 +10063,10 @@
       <c r="H44" s="29"/>
       <c r="I44" s="30"/>
       <c r="J44" s="178" t="s">
-        <v>357</v>
+        <v>359</v>
       </c>
       <c r="K44" s="28" t="s">
-        <v>358</v>
+        <v>360</v>
       </c>
       <c r="M44" s="53"/>
       <c r="N44" s="53"/>
@@ -9255,13 +10077,13 @@
     </row>
     <row r="45" ht="13.95" customHeight="1" spans="1:18">
       <c r="A45" s="25" t="s">
-        <v>332</v>
+        <v>334</v>
       </c>
       <c r="B45" s="52" t="s">
-        <v>386</v>
+        <v>388</v>
       </c>
       <c r="C45" s="27" t="s">
-        <v>387</v>
+        <v>389</v>
       </c>
       <c r="D45" s="27"/>
       <c r="E45" s="33"/>
@@ -9270,10 +10092,10 @@
       <c r="H45" s="29"/>
       <c r="I45" s="30"/>
       <c r="J45" s="178" t="s">
-        <v>357</v>
+        <v>359</v>
       </c>
       <c r="K45" s="28" t="s">
-        <v>358</v>
+        <v>360</v>
       </c>
       <c r="M45" s="53"/>
       <c r="N45" s="53"/>
@@ -9284,10 +10106,10 @@
     </row>
     <row r="46" ht="13.95" customHeight="1" spans="1:18">
       <c r="A46" s="25" t="s">
-        <v>332</v>
+        <v>334</v>
       </c>
       <c r="B46" s="52" t="s">
-        <v>388</v>
+        <v>390</v>
       </c>
       <c r="C46" s="27" t="s">
         <v>45</v>
@@ -9299,10 +10121,10 @@
       <c r="H46" s="29"/>
       <c r="I46" s="30"/>
       <c r="J46" s="178" t="s">
-        <v>357</v>
+        <v>359</v>
       </c>
       <c r="K46" s="28" t="s">
-        <v>358</v>
+        <v>360</v>
       </c>
       <c r="M46" s="53"/>
       <c r="N46" s="53"/>
@@ -9313,13 +10135,13 @@
     </row>
     <row r="47" ht="13.95" customHeight="1" spans="1:18">
       <c r="A47" s="25" t="s">
-        <v>332</v>
+        <v>334</v>
       </c>
       <c r="B47" s="52" t="s">
-        <v>316</v>
+        <v>318</v>
       </c>
       <c r="C47" s="27" t="s">
-        <v>317</v>
+        <v>319</v>
       </c>
       <c r="D47" s="27"/>
       <c r="E47" s="33"/>
@@ -9328,10 +10150,10 @@
       <c r="H47" s="29"/>
       <c r="I47" s="30"/>
       <c r="J47" s="178" t="s">
-        <v>357</v>
+        <v>359</v>
       </c>
       <c r="K47" s="28" t="s">
-        <v>358</v>
+        <v>360</v>
       </c>
       <c r="M47" s="53"/>
       <c r="N47" s="53"/>
@@ -9342,13 +10164,13 @@
     </row>
     <row r="48" ht="13.95" customHeight="1" spans="1:18">
       <c r="A48" s="25" t="s">
-        <v>332</v>
+        <v>334</v>
       </c>
       <c r="B48" s="52" t="s">
-        <v>389</v>
+        <v>391</v>
       </c>
       <c r="C48" s="27" t="s">
-        <v>390</v>
+        <v>392</v>
       </c>
       <c r="D48" s="27"/>
       <c r="E48" s="33"/>
@@ -9357,10 +10179,10 @@
       <c r="H48" s="29"/>
       <c r="I48" s="30"/>
       <c r="J48" s="178" t="s">
-        <v>357</v>
+        <v>359</v>
       </c>
       <c r="K48" s="28" t="s">
-        <v>358</v>
+        <v>360</v>
       </c>
       <c r="M48" s="53"/>
       <c r="N48" s="53"/>
@@ -9371,13 +10193,13 @@
     </row>
     <row r="49" ht="13.95" customHeight="1" spans="1:18">
       <c r="A49" s="25" t="s">
-        <v>332</v>
+        <v>334</v>
       </c>
       <c r="B49" s="52" t="s">
-        <v>391</v>
+        <v>393</v>
       </c>
       <c r="C49" s="27" t="s">
-        <v>392</v>
+        <v>394</v>
       </c>
       <c r="D49" s="27"/>
       <c r="E49" s="33"/>
@@ -9386,10 +10208,10 @@
       <c r="H49" s="29"/>
       <c r="I49" s="30"/>
       <c r="J49" s="178" t="s">
-        <v>357</v>
+        <v>359</v>
       </c>
       <c r="K49" s="28" t="s">
-        <v>358</v>
+        <v>360</v>
       </c>
       <c r="M49" s="53"/>
       <c r="N49" s="53"/>
@@ -9400,13 +10222,13 @@
     </row>
     <row r="50" ht="13.95" customHeight="1" spans="1:18">
       <c r="A50" s="25" t="s">
-        <v>332</v>
+        <v>334</v>
       </c>
       <c r="B50" s="52" t="s">
-        <v>393</v>
+        <v>395</v>
       </c>
       <c r="C50" s="27" t="s">
-        <v>394</v>
+        <v>396</v>
       </c>
       <c r="D50" s="27"/>
       <c r="E50" s="33"/>
@@ -9415,10 +10237,10 @@
       <c r="H50" s="29"/>
       <c r="I50" s="30"/>
       <c r="J50" s="178" t="s">
-        <v>357</v>
+        <v>359</v>
       </c>
       <c r="K50" s="28" t="s">
-        <v>358</v>
+        <v>360</v>
       </c>
       <c r="M50" s="53"/>
       <c r="N50" s="53"/>
@@ -9429,13 +10251,13 @@
     </row>
     <row r="51" ht="13.95" customHeight="1" spans="1:18">
       <c r="A51" s="25" t="s">
-        <v>332</v>
+        <v>334</v>
       </c>
       <c r="B51" s="52" t="s">
         <v>61</v>
       </c>
       <c r="C51" s="27" t="s">
-        <v>395</v>
+        <v>397</v>
       </c>
       <c r="D51" s="27"/>
       <c r="E51" s="33"/>
@@ -9444,10 +10266,10 @@
       <c r="H51" s="29"/>
       <c r="I51" s="30"/>
       <c r="J51" s="178" t="s">
-        <v>357</v>
+        <v>359</v>
       </c>
       <c r="K51" s="28" t="s">
-        <v>358</v>
+        <v>360</v>
       </c>
       <c r="M51" s="53"/>
       <c r="N51" s="53"/>
@@ -9458,13 +10280,13 @@
     </row>
     <row r="52" ht="13.95" customHeight="1" spans="1:18">
       <c r="A52" s="25" t="s">
-        <v>332</v>
+        <v>334</v>
       </c>
       <c r="B52" s="52" t="s">
-        <v>305</v>
+        <v>307</v>
       </c>
       <c r="C52" s="34" t="s">
-        <v>306</v>
+        <v>308</v>
       </c>
       <c r="D52" s="34"/>
       <c r="E52" s="33"/>
@@ -9473,10 +10295,10 @@
       <c r="H52" s="29"/>
       <c r="I52" s="30"/>
       <c r="J52" s="178" t="s">
-        <v>357</v>
+        <v>359</v>
       </c>
       <c r="K52" s="28" t="s">
-        <v>358</v>
+        <v>360</v>
       </c>
       <c r="M52" s="53"/>
       <c r="N52" s="53"/>
@@ -9487,13 +10309,13 @@
     </row>
     <row r="53" ht="13.95" customHeight="1" spans="1:18">
       <c r="A53" s="25" t="s">
-        <v>332</v>
+        <v>334</v>
       </c>
       <c r="B53" s="52" t="s">
-        <v>309</v>
+        <v>311</v>
       </c>
       <c r="C53" s="27" t="s">
-        <v>310</v>
+        <v>312</v>
       </c>
       <c r="D53" s="27"/>
       <c r="E53" s="33"/>
@@ -9502,10 +10324,10 @@
       <c r="H53" s="29"/>
       <c r="I53" s="30"/>
       <c r="J53" s="178" t="s">
-        <v>357</v>
+        <v>359</v>
       </c>
       <c r="K53" s="28" t="s">
-        <v>358</v>
+        <v>360</v>
       </c>
       <c r="M53" s="53"/>
       <c r="N53" s="53"/>
@@ -9516,13 +10338,13 @@
     </row>
     <row r="54" ht="13.95" customHeight="1" spans="1:18">
       <c r="A54" s="25" t="s">
-        <v>332</v>
+        <v>334</v>
       </c>
       <c r="B54" s="52" t="s">
-        <v>396</v>
+        <v>398</v>
       </c>
       <c r="C54" s="27" t="s">
-        <v>397</v>
+        <v>399</v>
       </c>
       <c r="D54" s="27"/>
       <c r="E54" s="33"/>
@@ -9531,10 +10353,10 @@
       <c r="H54" s="29"/>
       <c r="I54" s="30"/>
       <c r="J54" s="178" t="s">
-        <v>357</v>
+        <v>359</v>
       </c>
       <c r="K54" s="28" t="s">
-        <v>358</v>
+        <v>360</v>
       </c>
       <c r="M54" s="53"/>
       <c r="N54" s="53"/>
@@ -9545,13 +10367,13 @@
     </row>
     <row r="55" ht="13.95" customHeight="1" spans="1:18">
       <c r="A55" s="56" t="s">
-        <v>332</v>
+        <v>334</v>
       </c>
       <c r="B55" s="57" t="s">
-        <v>398</v>
+        <v>400</v>
       </c>
       <c r="C55" s="58" t="s">
-        <v>399</v>
+        <v>401</v>
       </c>
       <c r="D55" s="58"/>
       <c r="E55" s="59"/>
@@ -9560,10 +10382,10 @@
       <c r="H55" s="61"/>
       <c r="I55" s="62"/>
       <c r="J55" s="179" t="s">
-        <v>357</v>
+        <v>359</v>
       </c>
       <c r="K55" s="60" t="s">
-        <v>400</v>
+        <v>402</v>
       </c>
       <c r="M55" s="53"/>
       <c r="N55" s="53"/>
@@ -9574,13 +10396,13 @@
     </row>
     <row r="56" ht="13.95" customHeight="1" spans="1:18">
       <c r="A56" s="56" t="s">
-        <v>332</v>
+        <v>334</v>
       </c>
       <c r="B56" s="57" t="s">
-        <v>401</v>
+        <v>403</v>
       </c>
       <c r="C56" s="58" t="s">
-        <v>402</v>
+        <v>404</v>
       </c>
       <c r="D56" s="58"/>
       <c r="E56" s="59"/>
@@ -9592,7 +10414,7 @@
         <v>0</v>
       </c>
       <c r="K56" s="60" t="s">
-        <v>400</v>
+        <v>402</v>
       </c>
       <c r="M56" s="53"/>
       <c r="N56" s="53"/>
@@ -9658,10 +10480,10 @@
       <c r="D59" s="13"/>
       <c r="E59" s="21"/>
       <c r="F59" s="28" t="s">
-        <v>340</v>
+        <v>342</v>
       </c>
       <c r="G59" s="28" t="s">
-        <v>403</v>
+        <v>405</v>
       </c>
       <c r="H59" s="29" t="s">
         <v>109</v>
@@ -9716,7 +10538,7 @@
       <c r="D62" s="16"/>
       <c r="E62" s="16"/>
       <c r="F62" s="47" t="s">
-        <v>404</v>
+        <v>406</v>
       </c>
       <c r="G62" s="39"/>
       <c r="H62" s="39"/>
@@ -9728,7 +10550,7 @@
     <row r="63" ht="13.95" customHeight="1"/>
     <row r="64" ht="25" customHeight="1" spans="1:18">
       <c r="A64" s="14" t="s">
-        <v>284</v>
+        <v>286</v>
       </c>
       <c r="B64" s="15">
         <v>3</v>
@@ -9745,36 +10567,36 @@
     </row>
     <row r="65" ht="20" customHeight="1" spans="1:11">
       <c r="A65" s="17" t="s">
-        <v>405</v>
+        <v>407</v>
       </c>
       <c r="B65" s="12"/>
       <c r="C65" s="12"/>
       <c r="D65" s="13"/>
       <c r="E65" s="18"/>
       <c r="F65" s="19" t="s">
-        <v>286</v>
+        <v>288</v>
       </c>
       <c r="G65" s="19" t="s">
-        <v>406</v>
+        <v>408</v>
       </c>
       <c r="H65" s="13"/>
       <c r="I65" s="19" t="s">
-        <v>288</v>
+        <v>290</v>
       </c>
       <c r="J65" s="19" t="s">
-        <v>289</v>
+        <v>291</v>
       </c>
       <c r="K65" s="13"/>
     </row>
     <row r="66" ht="37" customHeight="1" spans="1:11">
       <c r="A66" s="20" t="s">
-        <v>294</v>
+        <v>296</v>
       </c>
       <c r="B66" s="20" t="s">
-        <v>295</v>
+        <v>297</v>
       </c>
       <c r="C66" s="20" t="s">
-        <v>296</v>
+        <v>298</v>
       </c>
       <c r="D66" s="20" t="s">
         <v>186</v>
@@ -9784,7 +10606,7 @@
         <v>40</v>
       </c>
       <c r="G66" s="23" t="s">
-        <v>297</v>
+        <v>299</v>
       </c>
       <c r="H66" s="23" t="s">
         <v>42</v>
@@ -9801,7 +10623,7 @@
     </row>
     <row r="67" ht="13.95" customHeight="1" spans="1:11">
       <c r="A67" s="25" t="s">
-        <v>282</v>
+        <v>284</v>
       </c>
       <c r="B67" s="52" t="s">
         <v>84</v>
@@ -9812,7 +10634,7 @@
       <c r="D67" s="34"/>
       <c r="E67" s="33"/>
       <c r="F67" s="28" t="s">
-        <v>332</v>
+        <v>334</v>
       </c>
       <c r="G67" s="28" t="s">
         <v>109</v>
@@ -9828,13 +10650,13 @@
     </row>
     <row r="68" ht="13.95" customHeight="1" spans="1:11">
       <c r="A68" s="25" t="s">
-        <v>282</v>
+        <v>284</v>
       </c>
       <c r="B68" s="52" t="s">
-        <v>334</v>
+        <v>336</v>
       </c>
       <c r="C68" s="27" t="s">
-        <v>335</v>
+        <v>337</v>
       </c>
       <c r="D68" s="27"/>
       <c r="E68" s="21"/>
@@ -9842,137 +10664,137 @@
       <c r="G68" s="28"/>
       <c r="H68" s="29"/>
       <c r="I68" s="30" t="s">
-        <v>336</v>
+        <v>338</v>
       </c>
       <c r="J68" s="28" t="s">
-        <v>337</v>
+        <v>339</v>
       </c>
       <c r="K68" s="28"/>
     </row>
     <row r="69" ht="13.95" customHeight="1" spans="1:11">
       <c r="A69" s="25" t="s">
-        <v>282</v>
+        <v>284</v>
       </c>
       <c r="B69" s="52" t="s">
-        <v>338</v>
+        <v>340</v>
       </c>
       <c r="C69" s="27" t="s">
-        <v>339</v>
+        <v>341</v>
       </c>
       <c r="D69" s="27"/>
       <c r="E69" s="31"/>
       <c r="F69" s="28" t="s">
-        <v>332</v>
+        <v>334</v>
       </c>
       <c r="G69" s="28" t="s">
         <v>109</v>
       </c>
       <c r="H69" s="52" t="s">
-        <v>338</v>
+        <v>340</v>
       </c>
       <c r="I69" s="27" t="s">
-        <v>339</v>
+        <v>341</v>
       </c>
       <c r="J69" s="28"/>
       <c r="K69" s="28"/>
     </row>
     <row r="70" ht="13.95" customHeight="1" spans="1:11">
       <c r="A70" s="25" t="s">
-        <v>282</v>
+        <v>284</v>
       </c>
       <c r="B70" s="52" t="s">
-        <v>343</v>
+        <v>345</v>
       </c>
       <c r="C70" s="34" t="s">
-        <v>344</v>
+        <v>346</v>
       </c>
       <c r="D70" s="34" t="s">
-        <v>345</v>
+        <v>347</v>
       </c>
       <c r="E70" s="31"/>
       <c r="F70" s="28" t="s">
-        <v>332</v>
+        <v>334</v>
       </c>
       <c r="G70" s="28" t="s">
         <v>109</v>
       </c>
       <c r="H70" s="52" t="s">
-        <v>343</v>
+        <v>345</v>
       </c>
       <c r="I70" s="34" t="s">
-        <v>344</v>
+        <v>346</v>
       </c>
       <c r="J70" s="28"/>
       <c r="K70" s="28"/>
     </row>
     <row r="71" ht="13.95" customHeight="1" spans="1:11">
       <c r="A71" s="25" t="s">
-        <v>282</v>
+        <v>284</v>
       </c>
       <c r="B71" s="52" t="s">
-        <v>347</v>
+        <v>349</v>
       </c>
       <c r="C71" s="34" t="s">
-        <v>348</v>
+        <v>350</v>
       </c>
       <c r="D71" s="34"/>
       <c r="E71" s="33"/>
       <c r="F71" s="28" t="s">
-        <v>332</v>
+        <v>334</v>
       </c>
       <c r="G71" s="28" t="s">
         <v>109</v>
       </c>
       <c r="H71" s="52" t="s">
-        <v>347</v>
+        <v>349</v>
       </c>
       <c r="I71" s="34" t="s">
-        <v>348</v>
+        <v>350</v>
       </c>
       <c r="J71" s="32"/>
       <c r="K71" s="28"/>
     </row>
     <row r="72" ht="13.95" customHeight="1" spans="1:11">
       <c r="A72" s="25" t="s">
-        <v>282</v>
+        <v>284</v>
       </c>
       <c r="B72" s="52" t="s">
-        <v>350</v>
+        <v>352</v>
       </c>
       <c r="C72" s="34" t="s">
-        <v>351</v>
+        <v>353</v>
       </c>
       <c r="D72" s="34"/>
       <c r="E72" s="33"/>
       <c r="F72" s="28" t="s">
-        <v>332</v>
+        <v>334</v>
       </c>
       <c r="G72" s="28" t="s">
         <v>109</v>
       </c>
       <c r="H72" s="52" t="s">
-        <v>350</v>
+        <v>352</v>
       </c>
       <c r="I72" s="34" t="s">
-        <v>351</v>
+        <v>353</v>
       </c>
       <c r="J72" s="28"/>
       <c r="K72" s="28"/>
     </row>
     <row r="73" ht="13.95" customHeight="1" spans="1:11">
       <c r="A73" s="25" t="s">
-        <v>282</v>
+        <v>284</v>
       </c>
       <c r="B73" s="52" t="s">
         <v>172</v>
       </c>
       <c r="C73" s="34" t="s">
-        <v>303</v>
+        <v>305</v>
       </c>
       <c r="D73" s="34"/>
       <c r="E73" s="33"/>
       <c r="F73" s="28" t="s">
-        <v>332</v>
+        <v>334</v>
       </c>
       <c r="G73" s="28" t="s">
         <v>109</v>
@@ -9981,25 +10803,25 @@
         <v>172</v>
       </c>
       <c r="I73" s="34" t="s">
-        <v>303</v>
+        <v>305</v>
       </c>
       <c r="J73" s="28"/>
       <c r="K73" s="28"/>
     </row>
     <row r="74" ht="13.95" customHeight="1" spans="1:11">
       <c r="A74" s="25" t="s">
-        <v>282</v>
+        <v>284</v>
       </c>
       <c r="B74" s="52" t="s">
         <v>170</v>
       </c>
       <c r="C74" s="34" t="s">
-        <v>352</v>
+        <v>354</v>
       </c>
       <c r="D74" s="34"/>
       <c r="E74" s="33"/>
       <c r="F74" s="28" t="s">
-        <v>332</v>
+        <v>334</v>
       </c>
       <c r="G74" s="28" t="s">
         <v>109</v>
@@ -10008,214 +10830,214 @@
         <v>170</v>
       </c>
       <c r="I74" s="34" t="s">
-        <v>352</v>
+        <v>354</v>
       </c>
       <c r="J74" s="28"/>
       <c r="K74" s="28"/>
     </row>
     <row r="75" ht="13.95" customHeight="1" spans="1:11">
       <c r="A75" s="25" t="s">
-        <v>282</v>
+        <v>284</v>
       </c>
       <c r="B75" s="52" t="s">
-        <v>353</v>
+        <v>355</v>
       </c>
       <c r="C75" s="34" t="s">
-        <v>354</v>
+        <v>356</v>
       </c>
       <c r="D75" s="34"/>
       <c r="E75" s="33"/>
       <c r="F75" s="28" t="s">
-        <v>332</v>
+        <v>334</v>
       </c>
       <c r="G75" s="28" t="s">
         <v>109</v>
       </c>
       <c r="H75" s="52" t="s">
-        <v>353</v>
+        <v>355</v>
       </c>
       <c r="I75" s="34" t="s">
-        <v>354</v>
+        <v>356</v>
       </c>
       <c r="J75" s="28"/>
       <c r="K75" s="28"/>
     </row>
     <row r="76" ht="13.95" customHeight="1" spans="1:11">
       <c r="A76" s="25" t="s">
-        <v>282</v>
+        <v>284</v>
       </c>
       <c r="B76" s="52" t="s">
-        <v>355</v>
+        <v>357</v>
       </c>
       <c r="C76" s="34" t="s">
-        <v>356</v>
+        <v>358</v>
       </c>
       <c r="D76" s="34"/>
       <c r="E76" s="33"/>
       <c r="F76" s="28" t="s">
-        <v>332</v>
+        <v>334</v>
       </c>
       <c r="G76" s="28" t="s">
         <v>109</v>
       </c>
       <c r="H76" s="52" t="s">
-        <v>355</v>
+        <v>357</v>
       </c>
       <c r="I76" s="34" t="s">
-        <v>356</v>
+        <v>358</v>
       </c>
       <c r="J76" s="28"/>
       <c r="K76" s="28"/>
     </row>
     <row r="77" ht="13.95" customHeight="1" spans="1:11">
       <c r="A77" s="25" t="s">
-        <v>282</v>
+        <v>284</v>
       </c>
       <c r="B77" s="52" t="s">
-        <v>359</v>
+        <v>361</v>
       </c>
       <c r="C77" s="34" t="s">
-        <v>360</v>
+        <v>362</v>
       </c>
       <c r="D77" s="34"/>
       <c r="E77" s="33"/>
       <c r="F77" s="28" t="s">
-        <v>332</v>
+        <v>334</v>
       </c>
       <c r="G77" s="28" t="s">
         <v>109</v>
       </c>
       <c r="H77" s="52" t="s">
-        <v>359</v>
+        <v>361</v>
       </c>
       <c r="I77" s="34" t="s">
-        <v>360</v>
+        <v>362</v>
       </c>
       <c r="J77" s="28"/>
       <c r="K77" s="28"/>
     </row>
     <row r="78" ht="13.95" customHeight="1" spans="1:11">
       <c r="A78" s="25" t="s">
-        <v>282</v>
+        <v>284</v>
       </c>
       <c r="B78" s="52" t="s">
-        <v>363</v>
+        <v>365</v>
       </c>
       <c r="C78" s="34" t="s">
-        <v>364</v>
+        <v>366</v>
       </c>
       <c r="D78" s="34"/>
       <c r="E78" s="33"/>
       <c r="F78" s="28" t="s">
-        <v>332</v>
+        <v>334</v>
       </c>
       <c r="G78" s="28" t="s">
         <v>109</v>
       </c>
       <c r="H78" s="52" t="s">
-        <v>363</v>
+        <v>365</v>
       </c>
       <c r="I78" s="34" t="s">
-        <v>364</v>
+        <v>366</v>
       </c>
       <c r="J78" s="28"/>
       <c r="K78" s="28"/>
     </row>
     <row r="79" ht="13.95" customHeight="1" spans="1:11">
       <c r="A79" s="25" t="s">
-        <v>282</v>
+        <v>284</v>
       </c>
       <c r="B79" s="52" t="s">
-        <v>367</v>
+        <v>369</v>
       </c>
       <c r="C79" s="34" t="s">
-        <v>368</v>
+        <v>370</v>
       </c>
       <c r="D79" s="34" t="s">
-        <v>369</v>
+        <v>371</v>
       </c>
       <c r="E79" s="33"/>
       <c r="F79" s="28" t="s">
-        <v>332</v>
+        <v>334</v>
       </c>
       <c r="G79" s="28" t="s">
         <v>109</v>
       </c>
       <c r="H79" s="52" t="s">
-        <v>367</v>
+        <v>369</v>
       </c>
       <c r="I79" s="34" t="s">
-        <v>368</v>
+        <v>370</v>
       </c>
       <c r="J79" s="28"/>
       <c r="K79" s="28"/>
     </row>
     <row r="80" ht="13.95" customHeight="1" spans="1:11">
       <c r="A80" s="25" t="s">
-        <v>282</v>
+        <v>284</v>
       </c>
       <c r="B80" s="52" t="s">
-        <v>371</v>
+        <v>373</v>
       </c>
       <c r="C80" s="34" t="s">
-        <v>372</v>
+        <v>374</v>
       </c>
       <c r="D80" s="34" t="s">
-        <v>373</v>
+        <v>375</v>
       </c>
       <c r="E80" s="33"/>
       <c r="F80" s="28" t="s">
-        <v>332</v>
+        <v>334</v>
       </c>
       <c r="G80" s="28" t="s">
         <v>109</v>
       </c>
       <c r="H80" s="52" t="s">
-        <v>371</v>
+        <v>373</v>
       </c>
       <c r="I80" s="34" t="s">
-        <v>372</v>
+        <v>374</v>
       </c>
       <c r="J80" s="28" t="s">
-        <v>374</v>
+        <v>376</v>
       </c>
       <c r="K80" s="28" t="s">
-        <v>407</v>
+        <v>409</v>
       </c>
     </row>
     <row r="81" ht="13.95" customHeight="1" spans="1:11">
       <c r="A81" s="25" t="s">
-        <v>282</v>
+        <v>284</v>
       </c>
       <c r="B81" s="52" t="s">
-        <v>375</v>
+        <v>377</v>
       </c>
       <c r="C81" s="34" t="s">
-        <v>376</v>
+        <v>378</v>
       </c>
       <c r="D81" s="34"/>
       <c r="E81" s="33"/>
       <c r="F81" s="28" t="s">
-        <v>332</v>
+        <v>334</v>
       </c>
       <c r="G81" s="28" t="s">
         <v>109</v>
       </c>
       <c r="H81" s="52" t="s">
-        <v>375</v>
+        <v>377</v>
       </c>
       <c r="I81" s="34" t="s">
-        <v>376</v>
+        <v>378</v>
       </c>
       <c r="J81" s="28"/>
       <c r="K81" s="28"/>
     </row>
     <row r="82" ht="13.95" customHeight="1" spans="1:11">
       <c r="A82" s="25" t="s">
-        <v>282</v>
+        <v>284</v>
       </c>
       <c r="B82" s="52" t="s">
-        <v>377</v>
+        <v>379</v>
       </c>
       <c r="C82" s="27" t="s">
         <v>212</v>
@@ -10223,13 +11045,13 @@
       <c r="D82" s="27"/>
       <c r="E82" s="33"/>
       <c r="F82" s="28" t="s">
-        <v>332</v>
+        <v>334</v>
       </c>
       <c r="G82" s="28" t="s">
         <v>109</v>
       </c>
       <c r="H82" s="52" t="s">
-        <v>377</v>
+        <v>379</v>
       </c>
       <c r="I82" s="27" t="s">
         <v>212</v>
@@ -10239,118 +11061,118 @@
     </row>
     <row r="83" ht="13.95" customHeight="1" spans="1:11">
       <c r="A83" s="25" t="s">
-        <v>282</v>
+        <v>284</v>
       </c>
       <c r="B83" s="52" t="s">
-        <v>380</v>
+        <v>382</v>
       </c>
       <c r="C83" s="27" t="s">
-        <v>381</v>
+        <v>383</v>
       </c>
       <c r="D83" s="27"/>
       <c r="E83" s="33"/>
       <c r="F83" s="28" t="s">
-        <v>332</v>
+        <v>334</v>
       </c>
       <c r="G83" s="28" t="s">
         <v>109</v>
       </c>
       <c r="H83" s="52" t="s">
-        <v>380</v>
+        <v>382</v>
       </c>
       <c r="I83" s="27" t="s">
-        <v>381</v>
+        <v>383</v>
       </c>
       <c r="J83" s="28"/>
       <c r="K83" s="28"/>
     </row>
     <row r="84" ht="13.95" customHeight="1" spans="1:11">
       <c r="A84" s="25" t="s">
-        <v>282</v>
+        <v>284</v>
       </c>
       <c r="B84" s="52" t="s">
-        <v>382</v>
+        <v>384</v>
       </c>
       <c r="C84" s="27" t="s">
-        <v>383</v>
+        <v>385</v>
       </c>
       <c r="D84" s="27"/>
       <c r="E84" s="33"/>
       <c r="F84" s="28" t="s">
-        <v>332</v>
+        <v>334</v>
       </c>
       <c r="G84" s="28" t="s">
         <v>109</v>
       </c>
       <c r="H84" s="52" t="s">
-        <v>382</v>
+        <v>384</v>
       </c>
       <c r="I84" s="27" t="s">
-        <v>383</v>
+        <v>385</v>
       </c>
       <c r="J84" s="28"/>
       <c r="K84" s="28"/>
     </row>
     <row r="85" ht="13.95" customHeight="1" spans="1:11">
       <c r="A85" s="25" t="s">
-        <v>282</v>
+        <v>284</v>
       </c>
       <c r="B85" s="52" t="s">
-        <v>384</v>
+        <v>386</v>
       </c>
       <c r="C85" s="27" t="s">
-        <v>385</v>
+        <v>387</v>
       </c>
       <c r="D85" s="27"/>
       <c r="E85" s="33"/>
       <c r="F85" s="28" t="s">
-        <v>332</v>
+        <v>334</v>
       </c>
       <c r="G85" s="28" t="s">
         <v>109</v>
       </c>
       <c r="H85" s="52" t="s">
-        <v>384</v>
+        <v>386</v>
       </c>
       <c r="I85" s="27" t="s">
-        <v>385</v>
+        <v>387</v>
       </c>
       <c r="J85" s="28"/>
       <c r="K85" s="28"/>
     </row>
     <row r="86" ht="13.95" customHeight="1" spans="1:11">
       <c r="A86" s="25" t="s">
-        <v>282</v>
+        <v>284</v>
       </c>
       <c r="B86" s="52" t="s">
-        <v>386</v>
+        <v>388</v>
       </c>
       <c r="C86" s="27" t="s">
-        <v>387</v>
+        <v>389</v>
       </c>
       <c r="D86" s="27"/>
       <c r="E86" s="33"/>
       <c r="F86" s="28" t="s">
-        <v>332</v>
+        <v>334</v>
       </c>
       <c r="G86" s="28" t="s">
         <v>109</v>
       </c>
       <c r="H86" s="52" t="s">
-        <v>386</v>
+        <v>388</v>
       </c>
       <c r="I86" s="27" t="s">
-        <v>387</v>
+        <v>389</v>
       </c>
       <c r="J86" s="28"/>
       <c r="K86" s="28"/>
     </row>
     <row r="87" ht="13.95" customHeight="1" spans="1:11">
       <c r="A87" s="25" t="s">
-        <v>282</v>
+        <v>284</v>
       </c>
       <c r="B87" s="52" t="s">
-        <v>388</v>
+        <v>390</v>
       </c>
       <c r="C87" s="27" t="s">
         <v>45</v>
@@ -10358,13 +11180,13 @@
       <c r="D87" s="27"/>
       <c r="E87" s="33"/>
       <c r="F87" s="28" t="s">
-        <v>332</v>
+        <v>334</v>
       </c>
       <c r="G87" s="28" t="s">
         <v>109</v>
       </c>
       <c r="H87" s="52" t="s">
-        <v>388</v>
+        <v>390</v>
       </c>
       <c r="I87" s="27" t="s">
         <v>45</v>
@@ -10374,126 +11196,126 @@
     </row>
     <row r="88" ht="13.95" customHeight="1" spans="1:11">
       <c r="A88" s="25" t="s">
-        <v>282</v>
+        <v>284</v>
       </c>
       <c r="B88" s="52" t="s">
-        <v>316</v>
+        <v>318</v>
       </c>
       <c r="C88" s="27" t="s">
-        <v>317</v>
+        <v>319</v>
       </c>
       <c r="D88" s="27"/>
       <c r="E88" s="33"/>
       <c r="F88" s="28" t="s">
-        <v>332</v>
+        <v>334</v>
       </c>
       <c r="G88" s="28" t="s">
         <v>109</v>
       </c>
       <c r="H88" s="52" t="s">
-        <v>316</v>
+        <v>318</v>
       </c>
       <c r="I88" s="27" t="s">
-        <v>317</v>
+        <v>319</v>
       </c>
       <c r="J88" s="28"/>
       <c r="K88" s="28"/>
     </row>
     <row r="89" ht="13.95" customHeight="1" spans="1:11">
       <c r="A89" s="25" t="s">
-        <v>282</v>
+        <v>284</v>
       </c>
       <c r="B89" s="52" t="s">
-        <v>389</v>
+        <v>391</v>
       </c>
       <c r="C89" s="27" t="s">
-        <v>390</v>
+        <v>392</v>
       </c>
       <c r="D89" s="27"/>
       <c r="E89" s="33"/>
       <c r="F89" s="28" t="s">
-        <v>332</v>
+        <v>334</v>
       </c>
       <c r="G89" s="28" t="s">
         <v>109</v>
       </c>
       <c r="H89" s="52" t="s">
-        <v>389</v>
+        <v>391</v>
       </c>
       <c r="I89" s="27" t="s">
-        <v>390</v>
+        <v>392</v>
       </c>
       <c r="J89" s="28"/>
       <c r="K89" s="28"/>
     </row>
     <row r="90" spans="1:11">
       <c r="A90" s="25" t="s">
-        <v>282</v>
+        <v>284</v>
       </c>
       <c r="B90" s="52" t="s">
-        <v>391</v>
+        <v>393</v>
       </c>
       <c r="C90" s="27" t="s">
-        <v>392</v>
+        <v>394</v>
       </c>
       <c r="D90" s="27"/>
       <c r="E90" s="33"/>
       <c r="F90" s="28" t="s">
-        <v>332</v>
+        <v>334</v>
       </c>
       <c r="G90" s="28" t="s">
         <v>109</v>
       </c>
       <c r="H90" s="52" t="s">
-        <v>391</v>
+        <v>393</v>
       </c>
       <c r="I90" s="27" t="s">
-        <v>392</v>
+        <v>394</v>
       </c>
       <c r="J90" s="28"/>
       <c r="K90" s="28"/>
     </row>
     <row r="91" spans="1:11">
       <c r="A91" s="25" t="s">
-        <v>282</v>
+        <v>284</v>
       </c>
       <c r="B91" s="52" t="s">
-        <v>393</v>
+        <v>395</v>
       </c>
       <c r="C91" s="27" t="s">
-        <v>394</v>
+        <v>396</v>
       </c>
       <c r="D91" s="27"/>
       <c r="E91" s="33"/>
       <c r="F91" s="28" t="s">
-        <v>332</v>
+        <v>334</v>
       </c>
       <c r="G91" s="28" t="s">
         <v>109</v>
       </c>
       <c r="H91" s="52" t="s">
-        <v>393</v>
+        <v>395</v>
       </c>
       <c r="I91" s="27" t="s">
-        <v>394</v>
+        <v>396</v>
       </c>
       <c r="J91" s="28"/>
       <c r="K91" s="28"/>
     </row>
     <row r="92" spans="1:11">
       <c r="A92" s="25" t="s">
-        <v>282</v>
+        <v>284</v>
       </c>
       <c r="B92" s="52" t="s">
         <v>61</v>
       </c>
       <c r="C92" s="27" t="s">
-        <v>395</v>
+        <v>397</v>
       </c>
       <c r="D92" s="27"/>
       <c r="E92" s="33"/>
       <c r="F92" s="28" t="s">
-        <v>332</v>
+        <v>334</v>
       </c>
       <c r="G92" s="28" t="s">
         <v>109</v>
@@ -10502,148 +11324,148 @@
         <v>61</v>
       </c>
       <c r="I92" s="27" t="s">
-        <v>395</v>
+        <v>397</v>
       </c>
       <c r="J92" s="28"/>
       <c r="K92" s="28"/>
     </row>
     <row r="93" spans="1:11">
       <c r="A93" s="25" t="s">
-        <v>282</v>
+        <v>284</v>
       </c>
       <c r="B93" s="52" t="s">
-        <v>305</v>
+        <v>307</v>
       </c>
       <c r="C93" s="34" t="s">
-        <v>306</v>
+        <v>308</v>
       </c>
       <c r="D93" s="34"/>
       <c r="E93" s="33"/>
       <c r="F93" s="28" t="s">
-        <v>332</v>
+        <v>334</v>
       </c>
       <c r="G93" s="28" t="s">
         <v>109</v>
       </c>
       <c r="H93" s="52" t="s">
-        <v>305</v>
+        <v>307</v>
       </c>
       <c r="I93" s="34" t="s">
-        <v>306</v>
+        <v>308</v>
       </c>
       <c r="J93" s="28"/>
       <c r="K93" s="28"/>
     </row>
     <row r="94" spans="1:11">
       <c r="A94" s="25" t="s">
-        <v>282</v>
+        <v>284</v>
       </c>
       <c r="B94" s="52" t="s">
-        <v>309</v>
+        <v>311</v>
       </c>
       <c r="C94" s="27" t="s">
-        <v>310</v>
+        <v>312</v>
       </c>
       <c r="D94" s="27"/>
       <c r="E94" s="33"/>
       <c r="F94" s="28" t="s">
-        <v>332</v>
+        <v>334</v>
       </c>
       <c r="G94" s="28" t="s">
         <v>109</v>
       </c>
       <c r="H94" s="52" t="s">
-        <v>309</v>
+        <v>311</v>
       </c>
       <c r="I94" s="27" t="s">
-        <v>310</v>
+        <v>312</v>
       </c>
       <c r="J94" s="28"/>
       <c r="K94" s="28"/>
     </row>
     <row r="95" spans="1:11">
       <c r="A95" s="25" t="s">
-        <v>282</v>
+        <v>284</v>
       </c>
       <c r="B95" s="52" t="s">
-        <v>396</v>
+        <v>398</v>
       </c>
       <c r="C95" s="27" t="s">
-        <v>397</v>
+        <v>399</v>
       </c>
       <c r="D95" s="27"/>
       <c r="E95" s="33"/>
       <c r="F95" s="28" t="s">
-        <v>332</v>
+        <v>334</v>
       </c>
       <c r="G95" s="28" t="s">
         <v>109</v>
       </c>
       <c r="H95" s="52" t="s">
-        <v>396</v>
+        <v>398</v>
       </c>
       <c r="I95" s="27" t="s">
-        <v>397</v>
+        <v>399</v>
       </c>
       <c r="J95" s="28"/>
       <c r="K95" s="28"/>
     </row>
     <row r="96" spans="1:11">
       <c r="A96" s="56" t="s">
-        <v>282</v>
+        <v>284</v>
       </c>
       <c r="B96" s="57" t="s">
-        <v>398</v>
+        <v>400</v>
       </c>
       <c r="C96" s="58" t="s">
-        <v>399</v>
+        <v>401</v>
       </c>
       <c r="D96" s="58"/>
       <c r="E96" s="59"/>
       <c r="F96" s="60" t="s">
-        <v>332</v>
+        <v>334</v>
       </c>
       <c r="G96" s="60" t="s">
         <v>109</v>
       </c>
       <c r="H96" s="57" t="s">
-        <v>396</v>
+        <v>398</v>
       </c>
       <c r="I96" s="58" t="s">
-        <v>399</v>
+        <v>401</v>
       </c>
       <c r="J96" s="60"/>
       <c r="K96" s="60" t="s">
-        <v>400</v>
+        <v>402</v>
       </c>
     </row>
     <row r="97" spans="1:11">
       <c r="A97" s="56" t="s">
-        <v>282</v>
+        <v>284</v>
       </c>
       <c r="B97" s="57" t="s">
-        <v>401</v>
+        <v>403</v>
       </c>
       <c r="C97" s="58" t="s">
-        <v>402</v>
+        <v>404</v>
       </c>
       <c r="D97" s="58"/>
       <c r="E97" s="59"/>
       <c r="F97" s="60" t="s">
-        <v>332</v>
+        <v>334</v>
       </c>
       <c r="G97" s="60" t="s">
         <v>109</v>
       </c>
       <c r="H97" s="57" t="s">
-        <v>401</v>
+        <v>403</v>
       </c>
       <c r="I97" s="58" t="s">
-        <v>402</v>
+        <v>404</v>
       </c>
       <c r="J97" s="60"/>
       <c r="K97" s="60" t="s">
-        <v>400</v>
+        <v>402</v>
       </c>
     </row>
     <row r="98" spans="1:11">
@@ -10697,10 +11519,10 @@
       <c r="D100" s="13"/>
       <c r="E100" s="21"/>
       <c r="F100" s="28" t="s">
-        <v>332</v>
+        <v>334</v>
       </c>
       <c r="G100" s="28" t="s">
-        <v>408</v>
+        <v>410</v>
       </c>
       <c r="H100" s="29" t="s">
         <v>109</v>
@@ -10744,7 +11566,7 @@
       <c r="D103" s="16"/>
       <c r="E103" s="16"/>
       <c r="F103" s="47" t="s">
-        <v>409</v>
+        <v>411</v>
       </c>
       <c r="G103" s="39"/>
       <c r="H103" s="39"/>
@@ -10754,7 +11576,7 @@
     </row>
     <row r="105" ht="22" customHeight="1" spans="1:11">
       <c r="A105" s="14" t="s">
-        <v>284</v>
+        <v>286</v>
       </c>
       <c r="B105" s="15">
         <v>4</v>
@@ -10771,36 +11593,36 @@
     </row>
     <row r="106" ht="27" customHeight="1" spans="1:11">
       <c r="A106" s="17" t="s">
-        <v>410</v>
+        <v>412</v>
       </c>
       <c r="B106" s="12"/>
       <c r="C106" s="12"/>
       <c r="D106" s="13"/>
       <c r="E106" s="18"/>
       <c r="F106" s="19" t="s">
-        <v>286</v>
+        <v>288</v>
       </c>
       <c r="G106" s="19" t="s">
-        <v>411</v>
+        <v>413</v>
       </c>
       <c r="H106" s="13"/>
       <c r="I106" s="19" t="s">
-        <v>288</v>
+        <v>290</v>
       </c>
       <c r="J106" s="19" t="s">
-        <v>412</v>
+        <v>414</v>
       </c>
       <c r="K106" s="13"/>
     </row>
     <row r="107" ht="25" customHeight="1" spans="1:11">
       <c r="A107" s="20" t="s">
-        <v>294</v>
+        <v>296</v>
       </c>
       <c r="B107" s="20" t="s">
-        <v>295</v>
+        <v>297</v>
       </c>
       <c r="C107" s="20" t="s">
-        <v>296</v>
+        <v>298</v>
       </c>
       <c r="D107" s="20" t="s">
         <v>186</v>
@@ -10810,7 +11632,7 @@
         <v>40</v>
       </c>
       <c r="G107" s="23" t="s">
-        <v>297</v>
+        <v>299</v>
       </c>
       <c r="H107" s="23" t="s">
         <v>42</v>
@@ -10827,16 +11649,16 @@
     </row>
     <row r="108" spans="1:11">
       <c r="A108" s="25" t="s">
-        <v>282</v>
+        <v>284</v>
       </c>
       <c r="B108" s="26" t="s">
-        <v>367</v>
+        <v>369</v>
       </c>
       <c r="C108" s="34" t="s">
-        <v>368</v>
+        <v>370</v>
       </c>
       <c r="D108" s="34" t="s">
-        <v>369</v>
+        <v>371</v>
       </c>
       <c r="E108" s="33"/>
       <c r="F108" s="28"/>
@@ -10844,51 +11666,51 @@
       <c r="H108" s="52"/>
       <c r="I108" s="34"/>
       <c r="J108" s="178" t="s">
-        <v>413</v>
+        <v>415</v>
       </c>
       <c r="K108" s="28"/>
     </row>
     <row r="109" spans="1:11">
       <c r="A109" s="25" t="s">
-        <v>282</v>
+        <v>284</v>
       </c>
       <c r="B109" s="26" t="s">
-        <v>316</v>
+        <v>318</v>
       </c>
       <c r="C109" s="27" t="s">
-        <v>317</v>
+        <v>319</v>
       </c>
       <c r="D109" s="27"/>
       <c r="E109" s="33"/>
       <c r="F109" s="28" t="s">
-        <v>298</v>
+        <v>300</v>
       </c>
       <c r="G109" s="28" t="s">
         <v>112</v>
       </c>
       <c r="H109" s="52" t="s">
-        <v>316</v>
+        <v>318</v>
       </c>
       <c r="I109" s="27" t="s">
-        <v>317</v>
+        <v>319</v>
       </c>
       <c r="J109" s="28"/>
       <c r="K109" s="28"/>
     </row>
     <row r="110" spans="1:11">
       <c r="A110" s="25" t="s">
-        <v>282</v>
+        <v>284</v>
       </c>
       <c r="B110" s="26" t="s">
         <v>61</v>
       </c>
       <c r="C110" s="27" t="s">
-        <v>395</v>
+        <v>397</v>
       </c>
       <c r="D110" s="27"/>
       <c r="E110" s="33"/>
       <c r="F110" s="28" t="s">
-        <v>298</v>
+        <v>300</v>
       </c>
       <c r="G110" s="28" t="s">
         <v>112</v>
@@ -10904,54 +11726,54 @@
     </row>
     <row r="111" spans="1:11">
       <c r="A111" s="25" t="s">
-        <v>282</v>
+        <v>284</v>
       </c>
       <c r="B111" s="26" t="s">
-        <v>305</v>
+        <v>307</v>
       </c>
       <c r="C111" s="34" t="s">
-        <v>306</v>
+        <v>308</v>
       </c>
       <c r="D111" s="34"/>
       <c r="E111" s="33"/>
       <c r="F111" s="28" t="s">
-        <v>298</v>
+        <v>300</v>
       </c>
       <c r="G111" s="28" t="s">
         <v>112</v>
       </c>
       <c r="H111" s="52" t="s">
-        <v>305</v>
+        <v>307</v>
       </c>
       <c r="I111" s="34" t="s">
-        <v>306</v>
+        <v>308</v>
       </c>
       <c r="J111" s="28"/>
       <c r="K111" s="28"/>
     </row>
     <row r="112" spans="1:11">
       <c r="A112" s="25" t="s">
-        <v>282</v>
+        <v>284</v>
       </c>
       <c r="B112" s="26" t="s">
-        <v>309</v>
+        <v>311</v>
       </c>
       <c r="C112" s="27" t="s">
-        <v>310</v>
+        <v>312</v>
       </c>
       <c r="D112" s="27"/>
       <c r="E112" s="33"/>
       <c r="F112" s="28" t="s">
-        <v>298</v>
+        <v>300</v>
       </c>
       <c r="G112" s="28" t="s">
         <v>112</v>
       </c>
       <c r="H112" s="52" t="s">
-        <v>309</v>
+        <v>311</v>
       </c>
       <c r="I112" s="27" t="s">
-        <v>310</v>
+        <v>312</v>
       </c>
       <c r="J112" s="28"/>
       <c r="K112" s="28"/>
@@ -11007,10 +11829,10 @@
       <c r="D115" s="13"/>
       <c r="E115" s="21"/>
       <c r="F115" s="28" t="s">
+        <v>284</v>
+      </c>
+      <c r="G115" s="28" t="s">
         <v>282</v>
-      </c>
-      <c r="G115" s="28" t="s">
-        <v>280</v>
       </c>
       <c r="H115" s="29" t="s">
         <v>109</v>
@@ -11026,17 +11848,17 @@
       <c r="D116" s="21"/>
       <c r="E116" s="21"/>
       <c r="F116" s="28" t="s">
-        <v>298</v>
+        <v>300</v>
       </c>
       <c r="G116" s="28" t="s">
-        <v>414</v>
+        <v>416</v>
       </c>
       <c r="H116" s="29" t="s">
         <v>112</v>
       </c>
       <c r="I116" s="30"/>
       <c r="J116" s="45" t="s">
-        <v>415</v>
+        <v>417</v>
       </c>
       <c r="K116" s="40"/>
     </row>
@@ -11088,7 +11910,7 @@
       <c r="D120" s="16"/>
       <c r="E120" s="16"/>
       <c r="F120" s="47" t="s">
-        <v>416</v>
+        <v>418</v>
       </c>
       <c r="G120" s="39"/>
       <c r="H120" s="39"/>
@@ -11186,7 +12008,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr codeName="Sheet690"/>
   <dimension ref="A1:D12"/>
@@ -11200,102 +12022,102 @@
   <sheetData>
     <row r="1" spans="1:4">
       <c r="A1" s="2" t="s">
-        <v>417</v>
+        <v>419</v>
       </c>
       <c r="B1" s="2" t="s">
         <v>33</v>
       </c>
       <c r="C1" s="2" t="s">
-        <v>418</v>
+        <v>420</v>
       </c>
       <c r="D1" s="2" t="s">
-        <v>419</v>
+        <v>421</v>
       </c>
     </row>
     <row r="2" spans="1:4">
       <c r="A2" s="2" t="s">
-        <v>420</v>
+        <v>422</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>421</v>
+        <v>423</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>422</v>
+        <v>424</v>
       </c>
       <c r="D2" s="2"/>
     </row>
     <row r="3" spans="1:4">
       <c r="A3" s="2" t="s">
-        <v>423</v>
+        <v>425</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>424</v>
+        <v>426</v>
       </c>
       <c r="C3" s="2" t="s">
-        <v>425</v>
+        <v>427</v>
       </c>
       <c r="D3" s="2"/>
     </row>
     <row r="4" spans="1:4">
       <c r="A4" s="2" t="s">
-        <v>426</v>
+        <v>428</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>427</v>
+        <v>429</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>428</v>
+        <v>430</v>
       </c>
       <c r="D4" s="2"/>
     </row>
     <row r="5" spans="1:4">
       <c r="A5" s="2" t="s">
-        <v>429</v>
+        <v>431</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>430</v>
+        <v>432</v>
       </c>
       <c r="C5" s="2" t="s">
-        <v>431</v>
+        <v>433</v>
       </c>
       <c r="D5" s="2"/>
     </row>
     <row r="6" spans="1:4">
       <c r="A6" s="2" t="s">
-        <v>432</v>
+        <v>434</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>433</v>
+        <v>435</v>
       </c>
       <c r="C6" s="2"/>
       <c r="D6" s="2"/>
     </row>
     <row r="7" spans="1:4">
       <c r="A7" s="2" t="s">
-        <v>434</v>
+        <v>436</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>435</v>
+        <v>437</v>
       </c>
       <c r="C7" s="2"/>
       <c r="D7" s="2"/>
     </row>
     <row r="8" spans="1:4">
       <c r="A8" s="2" t="s">
-        <v>436</v>
+        <v>438</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>437</v>
+        <v>439</v>
       </c>
       <c r="C8" s="2"/>
       <c r="D8" s="2"/>
     </row>
     <row r="9" spans="1:4">
       <c r="A9" s="2" t="s">
-        <v>438</v>
+        <v>440</v>
       </c>
       <c r="B9" s="2" t="s">
-        <v>439</v>
+        <v>441</v>
       </c>
       <c r="C9" s="2"/>
       <c r="D9" s="2"/>
@@ -11303,7 +12125,7 @@
     <row r="10" spans="1:4">
       <c r="A10" s="2"/>
       <c r="B10" s="2" t="s">
-        <v>440</v>
+        <v>442</v>
       </c>
       <c r="C10" s="2"/>
       <c r="D10" s="2"/>
@@ -11311,7 +12133,7 @@
     <row r="11" spans="1:4">
       <c r="A11" s="2"/>
       <c r="B11" s="2" t="s">
-        <v>441</v>
+        <v>443</v>
       </c>
       <c r="C11" s="2"/>
       <c r="D11" s="2"/>

</xml_diff>